<commit_message>
Momentum scan results 2026-10-11
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -1938,161 +1938,161 @@
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>VALU</t>
+          <t>RPGL</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>ARTW</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>FVNNU</t>
+          <t>TP</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>LSAK</t>
+          <t>ATOS</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>IRIX</t>
+          <t>JG</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>BTLN</t>
+          <t>AGBK</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>FEBO</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>BTSGU</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>SBC</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>ARTW</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>IDAI</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>JG</t>
+          <t>FEBO</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>BTSGU</t>
+          <t>LSAK</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>BTLN</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>AGBK</t>
+          <t>FVNNU</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>VALU</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>RPGL</t>
+          <t>IDAI</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>SMXT</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>IRIX</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-12
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A240"/>
+  <dimension ref="A1:A249"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,56 +426,56 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>ALISU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ACB</t>
+          <t>AACI</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AERO</t>
+          <t>LVLU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>ACHC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AZUL</t>
+          <t>AMBR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AEHL</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CRNT</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>DUO</t>
+          <t>AERO</t>
         </is>
       </c>
     </row>
@@ -489,14 +489,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>AHG</t>
+          <t>AEHL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>FBYD</t>
+          <t>BVFL</t>
         </is>
       </c>
     </row>
@@ -510,126 +510,126 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AIFA</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>HCAT</t>
+          <t>BMR</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BMR</t>
+          <t>AGBK</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>EMPD</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HRTX</t>
+          <t>CHNR</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>INSG</t>
+          <t>AIRT</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BPRE</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>LVLU</t>
+          <t>DLXY</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IRMD</t>
+          <t>AISP</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BRBI</t>
+          <t>INSG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>ELOG</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NTES</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ITRN</t>
+          <t>IRMD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AMBR</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Q</t>
+          <t>ITRN</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>FVNNU</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>QETA</t>
+          <t>AMPH</t>
         </is>
       </c>
     </row>
@@ -643,91 +643,91 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BWMN</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AMPH</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>LMB</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>LMB</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAPNU</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>SYPR</t>
+          <t>MYRG</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>NTCT</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>NTES</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>IDAI</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CCCT</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ANGI</t>
+          <t>OFLX</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OCG</t>
+          <t>LSAK</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
@@ -741,1358 +741,1421 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CLFD</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>APOG</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>OPTX</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>PWP</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>PEBK</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PWP</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CMRC</t>
+          <t>PWRL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>PWRL</t>
+          <t>QQQX</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>RFAI</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>RDGT</t>
+          <t>BIRD</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>BMNP</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ATRA</t>
+          <t>BPRE</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>FEAM</t>
+          <t>BRZE</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>FLD</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BWMN</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>GECCI</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>AXIN</t>
+          <t>CAPNU</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>GOOGM</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BGM</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>CDNS</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BLZR</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>CLMT</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CNXN</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>COPR</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CAMT</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CPHC</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IMKTA</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CELU</t>
+          <t>CRCT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CHEF</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>IPXG</t>
+          <t>CUB</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CLMB</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>CWCO</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CNXN</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>DMLP</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MTLS</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>DTST</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CURX</t>
+          <t>DUOL</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>NDSN</t>
+          <t>ECPG</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>NMAD</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CWCO</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>NTRP</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>ENSC</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DGII</t>
+          <t>EVCM</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>NVEC</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DMAC</t>
+          <t>FIRY</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>NXPL</t>
+          <t>FLXS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>DNMX</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>FOSL</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>ONBPP</t>
+          <t>FRD</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DTST</t>
+          <t>FROG</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>FSBW</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>DUOL</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EFOI</t>
+          <t>GECCH</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>GOOGM</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>PAX</t>
+          <t>GOOGN</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>PDSB</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>HBIO</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>PHUN</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>EUDA</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>PICS</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>HYFT</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>FCAP</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PSIG</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>FFIV</t>
+          <t>INAC</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>QQQX</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>FFR</t>
+          <t>INTR</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>QSI</t>
+          <t>IRIX</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>FIRY</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>JFU</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>RELL</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>FOSL</t>
+          <t>KE</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>RUSHB</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>KMRK</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>KRAQ</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>KRNT</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>KRSA</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>TLSA</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>LCUT</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>VAI</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>VCTR</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>ZSQR</t>
+          <t>LOPE</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>GOOGN</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>HQWWW</t>
+          <t>MSGM</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>NDSN</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KRNT</t>
+          <t>NECB</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>LCUT</t>
+          <t>NKSH</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LFCR</t>
+          <t>NMAD</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>NNBR</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>MACI</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>NTAP</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>NTGR</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>MBVI</t>
+          <t>NTRP</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MSGY</t>
+          <t>NXPL</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>ODD</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>OLLI</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>OM</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NTGR</t>
+          <t>ONBPP</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>OM</t>
+          <t>PAX</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>PBYI</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>PCB</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>PBYI</t>
+          <t>PDSB</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>PDFS</t>
+          <t>PICS</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>PKOH</t>
+          <t>PLUS</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>PNRG</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>PRHI</t>
+          <t>POCI</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PXS</t>
+          <t>PRDO</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>PRHI</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>PS</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>RFAI</t>
+          <t>PSIX</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>RIBBU</t>
+          <t>PUBM</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>RLYB</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>RRGB</t>
+          <t>RCKY</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>RDVT</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>RWAYL</t>
+          <t>RDWR</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>RGS</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>SAV</t>
+          <t>RMCF</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>SCSC</t>
+          <t>RVSB</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>SGC</t>
+          <t>RWAYM</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>SLAB</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>SOTK</t>
+          <t>SAMG</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>SSTI</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>STRK</t>
+          <t>SGC</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>SUJA</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>SKK</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>SWRD</t>
+          <t>SKWD</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>TJGC</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>TPCS</t>
+          <t>SMXT</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>TRNI</t>
+          <t>SNPS</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>SOTK</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>VIR</t>
+          <t>STDN</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>WCCB</t>
+          <t>STRA</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>XMTR</t>
+          <t>STRC</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>YDES</t>
+          <t>SVRN</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>RPGL</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>TACH</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>TP</t>
+          <t>TLN</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>TLSA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>JG</t>
+          <t>TPCS</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>AGBK</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>VAI</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>BTSGU</t>
+          <t>VCTR</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>SBC</t>
+          <t>WCCB</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>ARTW</t>
+          <t>BGM</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>SHLS</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>RELL</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>FEBO</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>LSAK</t>
+          <t>ZSQR</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>BTLN</t>
+          <t>RPGL</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>FVNNU</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>VALU</t>
+          <t>TEAM</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>IDAI</t>
+          <t>SUJA</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>SNWV</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>IRIX</t>
+          <t>GIBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>SWRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>RZLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>PGNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>KNSA</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>FLYW</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>STNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>MTEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>OLB</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>HQWWW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-14
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A228"/>
+  <dimension ref="A1:A193"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,1589 +426,1344 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AGBK</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>GFUZ</t>
+          <t>AHCO</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>ACHC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALISU</t>
+          <t>FNGR</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BCML</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CHNR</t>
+          <t>IMKTA</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADI</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>PFAI</t>
+          <t>ISPR</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DLHC</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>LIF</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>SIMA</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>EMPD</t>
+          <t>AGBK</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ELOG</t>
+          <t>AGCC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AIRT</t>
+          <t>AISP</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LVLU</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>AOUT</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>NXT</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FLYE</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ASTH</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PEBK</t>
+          <t>AUGO</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>RMCF</t>
+          <t>AVTR</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>AZTA</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>RPGL</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>BPRE</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>RSVR</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SNWV</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ARTW</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ATKR</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BKHAU</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>CLMT</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BMNP</t>
+          <t>CLOV</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>CRNC</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CLMB</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CMRC</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CNXN</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CORT</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CRCT</t>
+          <t>FEAM</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CRNC</t>
+          <t>FIVN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>FRPT</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>GIW</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>GOOGM</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>GOOGN</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>GRAL</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>EEIQ</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>IBRX</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>INTR</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>IRMD</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>FSBW</t>
+          <t>JFU</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>JRSH</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>GOOGM</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>GOOGN</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>KRNT</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>HMR</t>
+          <t>LCUT</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>LVLU</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>LYFT</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>MATH</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>IMPP</t>
+          <t>MDLN</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>MDXG</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IRMD</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>JANX</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KBON</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>KFFB</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>NMAD</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>NVAX</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>KROS</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>KRSA</t>
+          <t>OKTA</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>OLLI</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>PAX</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>LOCO</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>LOPE</t>
+          <t>PRHI</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>PRTH</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MCGA</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>MESH</t>
+          <t>QDEL</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>MGNI</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MNRO</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>RTSN</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>RZLT</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>NECB</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>NKSH</t>
+          <t>SANG</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>NXTC</t>
+          <t>SMXT</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>SND</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>OLLI</t>
+          <t>SOTK</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>SSNC</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>PANL</t>
+          <t>STNE</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>SWRD</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PDSB</t>
+          <t>TEAM</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PNRG</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>PRAA</t>
+          <t>VAI</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>VALU</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>WCCB</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>ELOG</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>PUBM</t>
+          <t>ODD</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>PXS</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>AIXI</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>QLEP</t>
+          <t>SUJA</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>RELL</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>QTEX</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>RFAI</t>
+          <t>BOLT</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>AHG</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>PDSB</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>KMRK</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SAMG</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SCSC</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>HEPS</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SLSN</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SMTI</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>ZSQR</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>SND</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>SNFCA</t>
+          <t>BMR</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>LOCO</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>SSTI</t>
+          <t>ENSC</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>PCRX</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>SUJA</t>
+          <t>BORR</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>PICS</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>SWRD</t>
+          <t>OPCH</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>PROF</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>TJGC</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>RPGL</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>FLYE</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>TW</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>WCCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>XFLH</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>ZSQR</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>AHG</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>FNKO</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>GCL</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>BYRN</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>MAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>APOG</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>JVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>HEPS</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>OKTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>SKWD</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>BRBI</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>AFYA</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>JG</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>BMR</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>PAYS</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>JDZG</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>RELL</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>SOTK</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>RCEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>NTSK</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>NAUT</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>PICS</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>AMPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>STNE</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>PRHI</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>IRIX</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>BRZE</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>LSAK</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>PAX</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>PBYI</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>FRSH</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-15
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A193"/>
+  <dimension ref="A1:A209"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,168 +426,168 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AHCO</t>
+          <t>AFRM</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACHC</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>FNGR</t>
+          <t>ACHC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>ATOS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>CLWT</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>IMKTA</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>AHG</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ISPR</t>
+          <t>GOOGM</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>CWCO</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LIF</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AFYA</t>
+          <t>AISP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGBK</t>
+          <t>FBYD</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AGCC</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>ANGH</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>RPGL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>RSVR</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ISPR</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>AOUT</t>
         </is>
       </c>
     </row>
@@ -601,1106 +601,1106 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ASTH</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>RZLT</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AUGO</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>AUGO</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AVTR</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BPRE</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>ATRA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>AUC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>BMBL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>BMNP</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>BLIV</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>BORR</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>BPRE</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>BREZ</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CLMT</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CLOV</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>CRNC</t>
+          <t>BTSGU</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CBFV</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>CBLL</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>CLGN</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>CRAC</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>FEAM</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>FRPT</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>FEAM</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>FERA</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>GIW</t>
+          <t>ECPG</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>FLYE</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>GOOGM</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>GOOGN</t>
+          <t>FRPT</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>GIW</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>IBRX</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>FAST</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>IRMD</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>JFU</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>IMKTA</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>GAINZ</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>KRNT</t>
+          <t>INTR</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>GECCI</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>LCUT</t>
+          <t>GILD</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>IRMD</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>LVLU</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>KRNT</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>IPXG</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MATH</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MDLN</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MDXG</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>JG</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>JRSH</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>MATH</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>MDLN</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>NMAD</t>
+          <t>KRSA</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>NVAX</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>OLLI</t>
+          <t>LVLU</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>MRNA</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>PAX</t>
+          <t>LYFT</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>PRHI</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>PAX</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>MCGA</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>PCRX</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>MSFT</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>RTSN</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>NMFCZ</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>PRTH</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>SANG</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>OKTA</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>OLLI</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SND</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>SOTK</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>RGCO</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>PACH</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>STNE</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SWRD</t>
+          <t>RTSN</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>PI</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>VAI</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>VALU</t>
+          <t>PRHI</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>WCCB</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ELOG</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>AIXI</t>
+          <t>SLSN</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>SUJA</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>RELL</t>
+          <t>SMXT</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>RWAYL</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>AHG</t>
+          <t>SND</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>PDSB</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>SOTK</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>STLD</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>SSNC</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>STNE</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>HEPS</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>SUJA</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ZSQR</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>TJGC</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>BMR</t>
+          <t>YDES</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>LOCO</t>
+          <t>ZSQR</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>VALU</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>CRNC</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>BORR</t>
+          <t>AHCO</t>
         </is>
       </c>
     </row>
@@ -1721,49 +1721,161 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PROF</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>KMRK</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>RPGL</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>FLYE</t>
+          <t>HEPS</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>HAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>JYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>QDEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>ELOG</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>AIXI</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>BRBI</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>HSTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>ENSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>GIBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>ODD</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>LOCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>HPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>PDSB</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>SHPH</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>APA</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>EZPW</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>CART</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-16
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A209"/>
+  <dimension ref="A1:A229"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,7 +433,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AFRM</t>
+          <t>FELE</t>
         </is>
       </c>
     </row>
@@ -447,623 +447,623 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ACHC</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AFYA</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>FLX</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CLWT</t>
+          <t>AHCO</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AIXI</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AHG</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GOOGM</t>
+          <t>FBYD</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CWCO</t>
+          <t>AMPH</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>FOIL</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>FBYD</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>AERO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ANGH</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>RPGL</t>
+          <t>PHUN</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>PNRG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>RSVR</t>
+          <t>AIRT</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ISPR</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>SOMN</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>RZLT</t>
+          <t>ASTH</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>AUGO</t>
+          <t>ATRA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>ANGI</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>AOUT</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ATRA</t>
+          <t>API</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AUC</t>
+          <t>AXIN</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BMBL</t>
+          <t>AZTA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>ASBH</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BMNP</t>
+          <t>BEBE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BLIV</t>
+          <t>BMR</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BORR</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BPRE</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BREZ</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BTSGU</t>
+          <t>BVFL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>CHPG</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>CMRC</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CBLL</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>CRAC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CBFV</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CBLL</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CLGN</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>DLXY</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CRAC</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>ELOG</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>ENSC</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>CNXN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>EVCM</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FEAM</t>
+          <t>FCBC</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>CRCT</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>FERA</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>ECPG</t>
+          <t>CRNC</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FLYE</t>
+          <t>FVNNU</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>FXAC</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FRPT</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GIW</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>GRAN</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>HOWL</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
@@ -1077,805 +1077,945 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IMKTA</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>GAINZ</t>
+          <t>EXFY</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>IMKTA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>GECCI</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>GILD</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IRMD</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>FRD</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>KRNT</t>
+          <t>LVLU</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IPXG</t>
+          <t>FWRG</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>MACI</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>GAING</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>GAINZ</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>JG</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MATH</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>GIBO</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MDLN</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>KRSA</t>
+          <t>MSGM</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>HBIO</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LVLU</t>
+          <t>NKSH</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>MRNA</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>NTES</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>HNNA</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>NXTC</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>PAX</t>
+          <t>OM</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MCGA</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>MSFT</t>
+          <t>IPXG</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PPLC</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>NMFCZ</t>
+          <t>PAX</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>PAYS</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>OKTA</t>
+          <t>PDSB</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>PFXNZ</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>OLLI</t>
+          <t>LOCO</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>LOPE</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>RGCO</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PACH</t>
+          <t>PRDO</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>RTSN</t>
+          <t>QQQX</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>PI</t>
+          <t>RTSN</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>RUSHB</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>PRHI</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>RVSB</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>RILYG</t>
+          <t>SAMG</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SLSN</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>RWAYL</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SND</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>SGC</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SOTK</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>SHPH</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>STNE</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>ODD</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>SUJA</t>
+          <t>SKWD</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>TJGC</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>YDES</t>
+          <t>SMPL</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>SMTI</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ZSQR</t>
+          <t>PBYI</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>VALU</t>
+          <t>SNFCA</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>CRNC</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>AHCO</t>
+          <t>SOTK</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>PICS</t>
+          <t>PCYO</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>SSTI</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>STRA</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>PRHI</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>HEPS</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>SWRD</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>PTLO</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ELOG</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>AIXI</t>
+          <t>TLN</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>BRBI</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>YDES</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>LOCO</t>
+          <t>RRGB</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>PDSB</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>SHPH</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>STRF</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>TASK</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>TBCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>TRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>QDEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>OXSQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>SUJA</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>HPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>FLYE</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>AHG</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>PICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>FRPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>JYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>JDZG</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>JZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>SMXT</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>AGBK</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>HSTM</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>KMRK</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>ICG</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>CRVL</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>BRBI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-17
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A229"/>
+  <dimension ref="A1:A153"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,70 +426,70 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>BHST</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>IA</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>CABR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FLX</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AHCO</t>
+          <t>AIXI</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AIXI</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>NDLS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FBYD</t>
+          <t>FOIL</t>
         </is>
       </c>
     </row>
@@ -503,21 +503,21 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>FOIL</t>
+          <t>AGBK</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
@@ -531,455 +531,455 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AERO</t>
+          <t>AGCC</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>AOUT</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>PHUN</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>ATOS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>PNRG</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AIRT</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>SOMN</t>
+          <t>AUGO</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ASTH</t>
+          <t>ASBH</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>BOLT</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>ATKR</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ATRA</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ANGI</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>BLMN</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>CDRO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AXIN</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ASBH</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BEBE</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BMR</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>ELOG</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>FELE</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CHPG</t>
+          <t>FRPT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CMRC</t>
+          <t>FSBW</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>GAING</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CRAC</t>
+          <t>GGR</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>DAAQ</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CBLL</t>
+          <t>DBCA</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>GRAN</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>DLXY</t>
+          <t>DMLP</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>DUKU</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>INBKZ</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ELOG</t>
+          <t>ETS</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>IRMD</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>JBDI</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CNXN</t>
+          <t>FCBC</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>EVCM</t>
+          <t>JCSE</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>FCBC</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CRCT</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>FOSL</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CRNC</t>
+          <t>FRHC</t>
         </is>
       </c>
     </row>
@@ -993,1029 +993,497 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>FXAC</t>
+          <t>LOPE</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>LVLU</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DHCNL</t>
+          <t>MATH</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GRAN</t>
+          <t>MSGM</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>NKSH</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>JG</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>OLB</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>LOCO</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>EXFY</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IMKTA</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>JANX</t>
+          <t>PDSB</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>PEBK</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FRD</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>RGCO</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>LVLU</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FWRG</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>MACI</t>
+          <t>RTSN</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GAING</t>
+          <t>RWAYM</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GAINZ</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>PTLO</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>SGRY</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>MSGM</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>HBIO</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>SKWD</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>SGC</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>NKSH</t>
+          <t>SMPL</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>NTES</t>
+          <t>SMXT</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>HNNA</t>
+          <t>SOMN</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>NXTC</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>OM</t>
+          <t>STLD</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>STRA</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>IPXG</t>
+          <t>SWRD</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>TDAY</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>XFLH</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>PAX</t>
+          <t>ODD</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>FWRG</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>PDSB</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>PFXNZ</t>
+          <t>PCRX</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>LOCO</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>SSEAU</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>LOPE</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>JZ</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>QQQX</t>
+          <t>GIBO</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>RILYG</t>
-        </is>
-      </c>
-    </row>
-    <row r="154">
-      <c r="A154" t="inlineStr">
-        <is>
-          <t>MEDP</t>
-        </is>
-      </c>
-    </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>RTSN</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>MKTX</t>
-        </is>
-      </c>
-    </row>
-    <row r="157">
-      <c r="A157" t="inlineStr">
-        <is>
-          <t>RUSHB</t>
-        </is>
-      </c>
-    </row>
-    <row r="158">
-      <c r="A158" t="inlineStr">
-        <is>
-          <t>MMSI</t>
-        </is>
-      </c>
-    </row>
-    <row r="159">
-      <c r="A159" t="inlineStr">
-        <is>
-          <t>RVSB</t>
-        </is>
-      </c>
-    </row>
-    <row r="160">
-      <c r="A160" t="inlineStr">
-        <is>
-          <t>MWYN</t>
-        </is>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>SAFT</t>
-        </is>
-      </c>
-    </row>
-    <row r="162">
-      <c r="A162" t="inlineStr">
-        <is>
-          <t>SAMG</t>
-        </is>
-      </c>
-    </row>
-    <row r="163">
-      <c r="A163" t="inlineStr">
-        <is>
-          <t>NCPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="164">
-      <c r="A164" t="inlineStr">
-        <is>
-          <t>SBAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="165">
-      <c r="A165" t="inlineStr">
-        <is>
-          <t>NRDS</t>
-        </is>
-      </c>
-    </row>
-    <row r="166">
-      <c r="A166" t="inlineStr">
-        <is>
-          <t>SCHL</t>
-        </is>
-      </c>
-    </row>
-    <row r="167">
-      <c r="A167" t="inlineStr">
-        <is>
-          <t>NSIT</t>
-        </is>
-      </c>
-    </row>
-    <row r="168">
-      <c r="A168" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-    </row>
-    <row r="169">
-      <c r="A169" t="inlineStr">
-        <is>
-          <t>SGC</t>
-        </is>
-      </c>
-    </row>
-    <row r="170">
-      <c r="A170" t="inlineStr">
-        <is>
-          <t>NTWK</t>
-        </is>
-      </c>
-    </row>
-    <row r="171">
-      <c r="A171" t="inlineStr">
-        <is>
-          <t>SHPH</t>
-        </is>
-      </c>
-    </row>
-    <row r="172">
-      <c r="A172" t="inlineStr">
-        <is>
-          <t>OCTV</t>
-        </is>
-      </c>
-    </row>
-    <row r="173">
-      <c r="A173" t="inlineStr">
-        <is>
-          <t>SIBN</t>
-        </is>
-      </c>
-    </row>
-    <row r="174">
-      <c r="A174" t="inlineStr">
-        <is>
-          <t>ODD</t>
-        </is>
-      </c>
-    </row>
-    <row r="175">
-      <c r="A175" t="inlineStr">
-        <is>
-          <t>SJ</t>
-        </is>
-      </c>
-    </row>
-    <row r="176">
-      <c r="A176" t="inlineStr">
-        <is>
-          <t>SKWD</t>
-        </is>
-      </c>
-    </row>
-    <row r="177">
-      <c r="A177" t="inlineStr">
-        <is>
-          <t>OSW</t>
-        </is>
-      </c>
-    </row>
-    <row r="178">
-      <c r="A178" t="inlineStr">
-        <is>
-          <t>SKYA</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" t="inlineStr">
-        <is>
-          <t>SMPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="180">
-      <c r="A180" t="inlineStr">
-        <is>
-          <t>SMTI</t>
-        </is>
-      </c>
-    </row>
-    <row r="181">
-      <c r="A181" t="inlineStr">
-        <is>
-          <t>PBYI</t>
-        </is>
-      </c>
-    </row>
-    <row r="182">
-      <c r="A182" t="inlineStr">
-        <is>
-          <t>SNFCA</t>
-        </is>
-      </c>
-    </row>
-    <row r="183">
-      <c r="A183" t="inlineStr">
-        <is>
-          <t>PCTY</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" t="inlineStr">
-        <is>
-          <t>SOTK</t>
-        </is>
-      </c>
-    </row>
-    <row r="185">
-      <c r="A185" t="inlineStr">
-        <is>
-          <t>PCYO</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" t="inlineStr">
-        <is>
-          <t>SPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" t="inlineStr">
-        <is>
-          <t>PNTG</t>
-        </is>
-      </c>
-    </row>
-    <row r="188">
-      <c r="A188" t="inlineStr">
-        <is>
-          <t>SSTI</t>
-        </is>
-      </c>
-    </row>
-    <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>PPLC</t>
-        </is>
-      </c>
-    </row>
-    <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>STRA</t>
-        </is>
-      </c>
-    </row>
-    <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>PRHI</t>
-        </is>
-      </c>
-    </row>
-    <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>SWKHL</t>
-        </is>
-      </c>
-    </row>
-    <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>PRVA</t>
-        </is>
-      </c>
-    </row>
-    <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>SWRD</t>
-        </is>
-      </c>
-    </row>
-    <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>PTLO</t>
-        </is>
-      </c>
-    </row>
-    <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>RCEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>TLN</t>
-        </is>
-      </c>
-    </row>
-    <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>RGC</t>
-        </is>
-      </c>
-    </row>
-    <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>TW</t>
-        </is>
-      </c>
-    </row>
-    <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>RPAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>RPD</t>
-        </is>
-      </c>
-    </row>
-    <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>YDES</t>
-        </is>
-      </c>
-    </row>
-    <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>RRGB</t>
-        </is>
-      </c>
-    </row>
-    <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>SLDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>SPSC</t>
-        </is>
-      </c>
-    </row>
-    <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>STLN</t>
-        </is>
-      </c>
-    </row>
-    <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>STRF</t>
-        </is>
-      </c>
-    </row>
-    <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>TASK</t>
-        </is>
-      </c>
-    </row>
-    <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>TBCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>TRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>QDEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>OXSQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>SUJA</t>
-        </is>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>HPK</t>
-        </is>
-      </c>
-    </row>
-    <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>FLYE</t>
-        </is>
-      </c>
-    </row>
-    <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
           <t>AHG</t>
-        </is>
-      </c>
-    </row>
-    <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>PICS</t>
-        </is>
-      </c>
-    </row>
-    <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>FRPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="219">
-      <c r="A219" t="inlineStr">
-        <is>
-          <t>JG</t>
-        </is>
-      </c>
-    </row>
-    <row r="220">
-      <c r="A220" t="inlineStr">
-        <is>
-          <t>JYD</t>
-        </is>
-      </c>
-    </row>
-    <row r="221">
-      <c r="A221" t="inlineStr">
-        <is>
-          <t>JDZG</t>
-        </is>
-      </c>
-    </row>
-    <row r="222">
-      <c r="A222" t="inlineStr">
-        <is>
-          <t>JZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="223">
-      <c r="A223" t="inlineStr">
-        <is>
-          <t>SMXT</t>
-        </is>
-      </c>
-    </row>
-    <row r="224">
-      <c r="A224" t="inlineStr">
-        <is>
-          <t>AGBK</t>
-        </is>
-      </c>
-    </row>
-    <row r="225">
-      <c r="A225" t="inlineStr">
-        <is>
-          <t>HSTM</t>
-        </is>
-      </c>
-    </row>
-    <row r="226">
-      <c r="A226" t="inlineStr">
-        <is>
-          <t>KMRK</t>
-        </is>
-      </c>
-    </row>
-    <row r="227">
-      <c r="A227" t="inlineStr">
-        <is>
-          <t>ICG</t>
-        </is>
-      </c>
-    </row>
-    <row r="228">
-      <c r="A228" t="inlineStr">
-        <is>
-          <t>CRVL</t>
-        </is>
-      </c>
-    </row>
-    <row r="229">
-      <c r="A229" t="inlineStr">
-        <is>
-          <t>BRBI</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-18
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -1378,70 +1378,70 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>FWRG</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>PCRX</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>FWRG</t>
+          <t>GIBO</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>AHG</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>SSEAU</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>SSEAU</t>
         </is>
       </c>
     </row>
@@ -1455,35 +1455,35 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>ODD</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>AHG</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-20
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A199"/>
+  <dimension ref="A1:A273"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,1386 +426,1904 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AERO</t>
+          <t>ABNB</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>AMSF</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BKYI</t>
+          <t>JCSE</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BIII</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>ASTH</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CABR</t>
+          <t>ACHC</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>AFYA</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>COCO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>ADSK</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>IOTR</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>ISPR</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>JZ</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>VAI</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FOIL</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>APOG</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>AMPH</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>INTJ</t>
+          <t>MELI</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IOTR</t>
+          <t>MGPI</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>MLKN</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>ANGI</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ARXS</t>
+          <t>ODFL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ASBH</t>
+          <t>OFIX</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>NDLS</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>APPF</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ATLO</t>
+          <t>PDD</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>AR</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BCML</t>
+          <t>PLAY</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>PWRL</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>PODD</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>ARXS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BLMN</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BMBL</t>
+          <t>QDEL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>SOLS</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>ATLO</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BWMN</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>TDAY</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>TRIP</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>AZN</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>COLM</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CPHC</t>
+          <t>BRBR</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CPOP</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>BSP</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>BVFL</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>BWMN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>CAI</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>CAQ</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>FACT</t>
+          <t>CBLL</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>FCBC</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>FLYE</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>CDW</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>FOSL</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>FRPT</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GAINI</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>CHYM</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>HWKN</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>COR</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>CSGP</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IPXG</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>JCSE</t>
+          <t>CTSH</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>LOPE</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>NAVN</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>NKSH</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>ENSC</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>NXPL</t>
+          <t>EVCM</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>OFRM</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>OLB</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>OM</t>
+          <t>EXPE</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>OXLCZ</t>
+          <t>FCBC</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>PEBK</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>PICS</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>FWRG</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>GEGGL</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>GEHC</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>PXS</t>
+          <t>GMAB</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>RGCO</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>RNW</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>HELE</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>RTSN</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>HUIZ</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>SAIH</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>SAMG</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>SCSC</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>SGC</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>SKWD</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>INTR</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>IPAR</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>STNE</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>SUJA</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>JVA</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>TILE</t>
+          <t>KDP</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>TRNZ</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>KMB</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>FWRG</t>
+          <t>LAUR</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>LFCR</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>OLLI</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>JG</t>
+          <t>MDLZ</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>SMPL</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ETS</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>MNRO</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>MRSH</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>PTLO</t>
+          <t>MTCH</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>NAVN</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>NCNO</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>PFAI</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>NTRSO</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>NWSA</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>ODD</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>OFRM</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>OFS</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>OLLI</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>OPCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>ORIQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>ORLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>OTEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>OXLCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>PEGA</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>PICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>PLGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>PRDO</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>PRVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>PTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>PTLO</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>PTON</t>
+        </is>
+      </c>
+    </row>
+    <row r="219">
+      <c r="A219" t="inlineStr">
+        <is>
+          <t>PYPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="220">
+      <c r="A220" t="inlineStr">
+        <is>
+          <t>QNBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="221">
+      <c r="A221" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="222">
+      <c r="A222" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="223">
+      <c r="A223" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="224">
+      <c r="A224" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" t="inlineStr">
+        <is>
+          <t>ROP</t>
+        </is>
+      </c>
+    </row>
+    <row r="226">
+      <c r="A226" t="inlineStr">
+        <is>
+          <t>ROST</t>
+        </is>
+      </c>
+    </row>
+    <row r="227">
+      <c r="A227" t="inlineStr">
+        <is>
+          <t>RPAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="228">
+      <c r="A228" t="inlineStr">
+        <is>
+          <t>RPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="229">
+      <c r="A229" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" t="inlineStr">
+        <is>
+          <t>RRGB</t>
+        </is>
+      </c>
+    </row>
+    <row r="231">
+      <c r="A231" t="inlineStr">
+        <is>
+          <t>RTSN</t>
+        </is>
+      </c>
+    </row>
+    <row r="232">
+      <c r="A232" t="inlineStr">
+        <is>
+          <t>RVSB</t>
+        </is>
+      </c>
+    </row>
+    <row r="233">
+      <c r="A233" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="234">
+      <c r="A234" t="inlineStr">
+        <is>
+          <t>SGRY</t>
+        </is>
+      </c>
+    </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>SHOO</t>
+        </is>
+      </c>
+    </row>
+    <row r="236">
+      <c r="A236" t="inlineStr">
+        <is>
+          <t>SHOP</t>
+        </is>
+      </c>
+    </row>
+    <row r="237">
+      <c r="A237" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+    </row>
+    <row r="238">
+      <c r="A238" t="inlineStr">
+        <is>
+          <t>SKWD</t>
+        </is>
+      </c>
+    </row>
+    <row r="239">
+      <c r="A239" t="inlineStr">
+        <is>
+          <t>SKYA</t>
+        </is>
+      </c>
+    </row>
+    <row r="240">
+      <c r="A240" t="inlineStr">
+        <is>
+          <t>SLDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="241">
+      <c r="A241" t="inlineStr">
+        <is>
+          <t>SNFCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="242">
+      <c r="A242" t="inlineStr">
+        <is>
+          <t>SPSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="243">
+      <c r="A243" t="inlineStr">
+        <is>
+          <t>SPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="244">
+      <c r="A244" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="245">
+      <c r="A245" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="246">
+      <c r="A246" t="inlineStr">
+        <is>
+          <t>STNE</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>STRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>SZZL</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>TEAM</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>TRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>VAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>XZO</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>YSWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>BLMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>CBRL</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>DCBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>JG</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>BYRN</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>TBCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>JDZG</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>MXCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>JBDI</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>IDXX</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>BMBL</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>TCRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>JYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>HPK</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-21
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A273"/>
+  <dimension ref="A1:A277"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -433,1897 +433,1925 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>JCSE</t>
+          <t>ACHC</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>ATAT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASTH</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACHC</t>
+          <t>AZN</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>COCO</t>
+          <t>ADSK</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>CHDN</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>CROX</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>CSX</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>IOTR</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>ENSG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ISPR</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AFYA</t>
+          <t>EXC</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>JZ</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>FLX</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>FSV</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMPH</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>MELI</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>KWY</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>APPF</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>LNT</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>MLKN</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ANGI</t>
+          <t>ODFL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>OFIX</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>OXSQ</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>APPF</t>
+          <t>PECO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>ASBH</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>PWRL</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>PDD</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AR</t>
+          <t>QDEL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>SOLS</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>AUDC</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ARXS</t>
+          <t>TCMD</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>PPLC</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>AVTR</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>BCML</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ATLO</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>BRBR</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>BSVN</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>TDAY</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>BTSG</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TRIP</t>
+          <t>BVS</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>CAI</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>CAKE</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>CART</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BRBR</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>CBLL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BSP</t>
+          <t>CDW</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BWMN</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>CHYM</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>CMRC</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CAQ</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CBLL</t>
+          <t>CSGP</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>CTSH</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>DLO</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CHYM</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>COR</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>EXFY</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>EZPW</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>FAST</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>GABC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GMAB</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>HOWL</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>EVCM</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>IA</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>IGAC</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>FCBC</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>FWRG</t>
+          <t>IPAR</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>IRMD</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>GEGGL</t>
+          <t>JCAP</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>LOCO</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>HELE</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>HUIZ</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>HWKN</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>INTR</t>
+          <t>MNRO</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>MRSH</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>NAUT</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>NAVN</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>NCNO</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>KDP</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>LAUR</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>LFCR</t>
+          <t>NXPL</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>ODD</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>OFRM</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>OLB</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>ONC</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>MDLZ</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>PAA</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MNRO</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>PAYS</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>MRSH</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>MTCH</t>
+          <t>PMTS</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>PODD</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NAVN</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>NCNO</t>
+          <t>PRME</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>PSIX</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>PTLE</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>PYPL</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>RCKY</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>OFRM</t>
+          <t>REAL</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>OFS</t>
+          <t>REF</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>OLLI</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>RELY</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>ORIQ</t>
+          <t>RGCO</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>ORLY</t>
+          <t>ROOT</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>ROST</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>OXLCM</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>PEGA</t>
+          <t>RTSN</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>PICS</t>
+          <t>RVSB</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>SHOP</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>PTLO</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>SJ</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>SKIN</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>SMPL</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>SNFCA</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>SSTI</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>SUNB</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>RRGB</t>
+          <t>TASK</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>RTSN</t>
+          <t>TCRT</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>TEAM</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>TENB</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>SGRY</t>
+          <t>TLN</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>SHOO</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>SKWD</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>VYLR</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>WLTH</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>SNFCA</t>
+          <t>WSBCO</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>XZO</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>YMAT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>SSTI</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>STNE</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>STRA</t>
+          <t>HUIZ</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>KMB</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>SZZL</t>
+          <t>BMBL</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>ERIC</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>IRLA</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>VAI</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>XZO</t>
+          <t>EVER</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>MTC</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>BLMN</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>JG</t>
+          <t>JBDI</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>PAYX</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>JRVR</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>JBDI</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>ETS</t>
+          <t>DH</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>EXPE</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>BMBL</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>TCRT</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>SSNC</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>BR</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>HCM</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>LYFT</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>HLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>WTW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-22
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A277"/>
+  <dimension ref="A1:A295"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,434 +426,434 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ABNB</t>
+          <t>AMSF</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACHC</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ATAT</t>
+          <t>ADBE</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>FLX</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ADSK</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>GIII</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>GPGI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CROX</t>
+          <t>IOTR</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>CSX</t>
+          <t>KLTR</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>LIF</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>FLX</t>
+          <t>MGPI</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>FSV</t>
+          <t>NXGL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>ODFL</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>APOG</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>OSG</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>APPF</t>
+          <t>AMPH</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>PODD</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>REYN</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>OXSQ</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>AOUT</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>TRIP</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ASBH</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>PWRL</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>ATLO</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>AVTR</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>AZN</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TCMD</t>
+          <t>BANF</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>BCML</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BFST</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BCML</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BRBR</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BTSG</t>
+          <t>BRZE</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BVS</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>BSVN</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>BVS</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CAKE</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CBLL</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
@@ -888,35 +888,35 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
@@ -930,1428 +930,1554 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CHYM</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CMRC</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>CPIX</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CSGP</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>CTSH</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>CYRX</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DLO</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>DMAC</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>DMLP</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>DUKU</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>EXFY</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>ENSC</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>EZPW</t>
+          <t>ESLT</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>FAST</t>
+          <t>ETSY</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>EVAX</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>EVER</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>EXC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>EXE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>FRSH</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>FSV</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>GMAB</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IGAC</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>HCM</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IRMD</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>JCAP</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>LOCO</t>
+          <t>IDXX</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>IRMD</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>JRSH</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>MNRO</t>
+          <t>KIDS</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>KMB</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MRSH</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>NAVN</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>NCNO</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>LNT</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>LOPE</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>MAT</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>MICC</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>NXPL</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>ODD</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>OFRM</t>
+          <t>MNST</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>OLB</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>MRSH</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>MZTI</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>NAUT</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>NAVN</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>NCNO</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>PAYS</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>PMTS</t>
+          <t>NECB</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>NTRSO</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>PSIX</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>NWSA</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PTLE</t>
+          <t>OCCIM</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>OFS</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>RCKY</t>
+          <t>ORIC</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>REF</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>OTTR</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>RGCO</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>ROOT</t>
+          <t>PAGP</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>ROST</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>PAYX</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>PBYI</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>RTSN</t>
+          <t>PCRX</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>PEP</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>SBAC</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>SHOP</t>
+          <t>PLUS</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>PMTS</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>POWW</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>SJ</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>SKIN</t>
+          <t>PRTH</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>PRVA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>SMPL</t>
+          <t>PYPL</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>SNFCA</t>
+          <t>QDEL</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>SSTI</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>ROOT</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>TASK</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>TCRT</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>TLN</t>
+          <t>RUSHB</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>SBUX</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>VYLR</t>
+          <t>SEIC</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>WLTH</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>WSBCO</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>XZO</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>YMAT</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>SMXT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>HUIZ</t>
+          <t>SSNC</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>BMBL</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>TASK</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>TCPC</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>TCRT</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>IRLA</t>
+          <t>TEAM</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>TENB</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>EVER</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>MTC</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>TRXB</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>JBDI</t>
+          <t>VAI</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>VSXY</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>WLTH</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>JRVR</t>
+          <t>XZO</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>DH</t>
+          <t>BTOC</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>EXPE</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>PEPG</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>OPK</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>LYFT</t>
+          <t>BMBL</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>BLMN</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>LOGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>NRIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>JDZG</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>INDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>KPLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>ENTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>MAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>RGC</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>ETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>SKYA</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>ARQT</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>SKIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>RTSN</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>ASO</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>HUIZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>JRVR</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>DH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-23
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A295"/>
+  <dimension ref="A1:A290"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,210 +426,210 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>AGNT</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ADBE</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AMSF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>FLX</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>ENSG</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>BRBR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>FRPT</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>CHNR</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>IOTR</t>
+          <t>ADSK</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AFYA</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>KLTR</t>
+          <t>GIII</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>DPZ</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>GPGI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>LIF</t>
+          <t>FLX</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>APEI</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>NXGL</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>IPAR</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>ODFL</t>
+          <t>KLTR</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>KWY</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>AMPH</t>
+          <t>LIF</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>ASBP</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>MGPI</t>
         </is>
       </c>
     </row>
@@ -643,224 +643,224 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>REYN</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>NXGL</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>ANGI</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>ATOS</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TRIP</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>APOG</t>
+          <t>REYN</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>TILE</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>SHOE</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ATLO</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AVTR</t>
+          <t>ASBH</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>BREZ</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>BANF</t>
+          <t>TCMD</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BCML</t>
+          <t>TRIB</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>BFST</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>TRIP</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>ATLO</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>BVFL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BRZE</t>
+          <t>BANF</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>BCAL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>BYRN</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BVS</t>
+          <t>BCML</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CART</t>
+          <t>BFST</t>
         </is>
       </c>
     </row>
@@ -874,280 +874,280 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CLAR</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>CHDN</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>BSVN</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CPIX</t>
+          <t>BVS</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>COLM</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>CBFV</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CSGP</t>
+          <t>CPIX</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CCNEP</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>DDI</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>DGICA</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>CHCO</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DMAC</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>DRDB</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DUKU</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>CRAC</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>ENSC</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
@@ -1161,1274 +1161,1274 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ETSY</t>
+          <t>EYE</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>EVAX</t>
+          <t>CWST</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>EVER</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>DAVE</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>DMAA</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>FOX</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>DSGR</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>FVN</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>DUKU</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FRSH</t>
+          <t>GABC</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>FSV</t>
+          <t>ECCU</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GMAB</t>
+          <t>GP</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>HCM</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>HUIZ</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>EVCM</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>IDXX</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>EVER</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>JRSH</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>JVA</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>FERAU</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>KTWO</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>FORR</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>IRMD</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>FSV</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>KINS</t>
+          <t>MICC</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KMB</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>NKSH</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>LOPE</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>NWS</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>OCCIM</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>OFIX</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MICC</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MNST</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MRSH</t>
+          <t>OTTR</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>PEPG</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>NAVN</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>NCNO</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>PLUS</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>NECB</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>PRDO</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>NWSA</t>
+          <t>PTON</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>OCCIM</t>
+          <t>KIDS</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>OFS</t>
+          <t>RGCO</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>ROOT</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>RWAYI</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>OTTR</t>
+          <t>RWAYL</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>SAMG</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>LOPE</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>PBYI</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>SOMN</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>PEP</t>
+          <t>STGW</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>STLN</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>TASK</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>PMTS</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>TCPC</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>TCRT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>MTC</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>PYPL</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>TRAD</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>TRAX</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>MZTI</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>ROOT</t>
+          <t>TRXB</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>VAI</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>WLTH</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>NCPL</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>NECB</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>RUSHB</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>OLED</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>SBUX</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>SEIC</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>PBYI</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>PCB</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>SMXT</t>
+          <t>PLBC</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>POWW</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>RCKY</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>TASK</t>
+          <t>REF</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>TCPC</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>TCRT</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>TEAM</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>SBC</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>TRXB</t>
+          <t>SBFG</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>SDHIU</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>SEIC</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>VAI</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>VSXY</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>WLTH</t>
+          <t>SKWD</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>XZO</t>
+          <t>SMPL</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>BTOC</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>TONT</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>TRS</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>XZO</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>OPK</t>
+          <t>ETS</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>BMBL</t>
+          <t>JRVR</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>BLMN</t>
+          <t>BMBL</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>ORIC</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>BLMN</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>OPK</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>ETS</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>PTLE</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
@@ -2443,41 +2443,6 @@
       <c r="A290" t="inlineStr">
         <is>
           <t>RTSN</t>
-        </is>
-      </c>
-    </row>
-    <row r="291">
-      <c r="A291" t="inlineStr">
-        <is>
-          <t>ASO</t>
-        </is>
-      </c>
-    </row>
-    <row r="292">
-      <c r="A292" t="inlineStr">
-        <is>
-          <t>OLED</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" t="inlineStr">
-        <is>
-          <t>HUIZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="294">
-      <c r="A294" t="inlineStr">
-        <is>
-          <t>JRVR</t>
-        </is>
-      </c>
-    </row>
-    <row r="295">
-      <c r="A295" t="inlineStr">
-        <is>
-          <t>DH</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-24
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A290"/>
+  <dimension ref="A1:A247"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,2023 +426,1722 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>AGBK</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>AGNT</t>
+          <t>ABLV</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>BHST</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>AQB</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>ADAMI</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>BVC</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BRBR</t>
+          <t>ASR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>AIIR</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>FRPT</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>CHNR</t>
+          <t>AIXI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>AFYA</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>EJH</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>LFS</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>DPZ</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>AHG</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GPGI</t>
+          <t>GIII</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>FLX</t>
+          <t>AMRO</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>GRFS</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>APEI</t>
+          <t>OSG</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>APOG</t>
+          <t>PLBY</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KLTR</t>
+          <t>KWY</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>PODD</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>LIF</t>
+          <t>MIDD</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ASBP</t>
+          <t>RGC</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>BETR</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>PEPG</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>NXGL</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ANGI</t>
+          <t>BMBL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ATOS</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>TCMD</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>REYN</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>TILE</t>
+          <t>BVFL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>SHOE</t>
+          <t>BDCI</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>BOLT</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ASBH</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BREZ</t>
+          <t>BOTJ</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>TCMD</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>TRIB</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>BRBI</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>TRIP</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>ATLO</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BANF</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BCAL</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>BYRN</t>
+          <t>CBFV</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BCML</t>
+          <t>CPIX</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>CWST</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BFST</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CCSI</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>DMAC</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>DRDB</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BVS</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>COLM</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CPIX</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>FUNC</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>GAING</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CCNEP</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>GAINI</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DDI</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>GAINZ</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>DGICA</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DHCNL</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DIBS</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CLAR</t>
+          <t>ETS</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DRDB</t>
+          <t>HEPS</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>HOWL</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CRAC</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>HUIZ</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>FORR</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>EYE</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CWST</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>DAVE</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>IPXG</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>DMAA</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FOX</t>
+          <t>JCSE</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DSGR</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>FVN</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DUKU</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>ECCU</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GP</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>HCM</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>MBRX</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>HUIZ</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>EVCM</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>MMTX</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>EVER</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>MTLS</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>JRSH</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>NPAC</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>FERAU</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>KTWO</t>
+          <t>NWFL</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>ONBPP</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>FORR</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>ONC</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>MGYR</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FSV</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>OTLY</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>OXLCZ</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>MICC</t>
+          <t>PAX</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>PCRX</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>NAUT</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>NKSH</t>
+          <t>PICS</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>PMTS</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>NWS</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>OCCIM</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>NSSC</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>PTLE</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>NTRSO</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>REBN</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>REVB</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>HWKN</t>
+          <t>OABI</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>OTTR</t>
+          <t>RIGL</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HYNE</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>RVSB</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>RWAYI</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>ORIC</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>PPLC</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>TBCH</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>POWW</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>PRDO</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>TRAX</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>PRME</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>PSIG</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>RGCO</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>KINS</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ROOT</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>REAL</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>REF</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>RWAYI</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>RWAYL</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>SAMG</t>
+          <t>SBFG</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>LOPE</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>LSBK</t>
+          <t>TACO</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>SOMN</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>STGW</t>
+          <t>CAPS</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>DGICB</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>TASK</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>AEYE</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>TCPC</t>
+          <t>OMH</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>TCRT</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>MTC</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>ALGN</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>TRAD</t>
+          <t>SVIAW</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>TRAX</t>
+          <t>EVAX</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>TRXB</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>VAI</t>
+          <t>MTEX</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>WLTH</t>
+          <t>BMGL</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>NCPL</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>NECB</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>OLED</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>JRVR</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>SLE</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>PAHC</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>PBYI</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>EXYN</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>PLBC</t>
+          <t>GP</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>OPK</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>POWW</t>
-        </is>
-      </c>
-    </row>
-    <row r="248">
-      <c r="A248" t="inlineStr">
-        <is>
-          <t>QNBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="249">
-      <c r="A249" t="inlineStr">
-        <is>
-          <t>RCEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="250">
-      <c r="A250" t="inlineStr">
-        <is>
-          <t>RCKY</t>
-        </is>
-      </c>
-    </row>
-    <row r="251">
-      <c r="A251" t="inlineStr">
-        <is>
-          <t>REF</t>
-        </is>
-      </c>
-    </row>
-    <row r="252">
-      <c r="A252" t="inlineStr">
-        <is>
-          <t>REGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="253">
-      <c r="A253" t="inlineStr">
-        <is>
-          <t>ROP</t>
-        </is>
-      </c>
-    </row>
-    <row r="254">
-      <c r="A254" t="inlineStr">
-        <is>
-          <t>RPAY</t>
-        </is>
-      </c>
-    </row>
-    <row r="255">
-      <c r="A255" t="inlineStr">
-        <is>
-          <t>RPD</t>
-        </is>
-      </c>
-    </row>
-    <row r="256">
-      <c r="A256" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="257">
-      <c r="A257" t="inlineStr">
-        <is>
-          <t>SBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="258">
-      <c r="A258" t="inlineStr">
-        <is>
-          <t>SBFG</t>
-        </is>
-      </c>
-    </row>
-    <row r="259">
-      <c r="A259" t="inlineStr">
-        <is>
-          <t>SDHIU</t>
-        </is>
-      </c>
-    </row>
-    <row r="260">
-      <c r="A260" t="inlineStr">
-        <is>
-          <t>SEIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="261">
-      <c r="A261" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-    </row>
-    <row r="262">
-      <c r="A262" t="inlineStr">
-        <is>
-          <t>SIGI</t>
-        </is>
-      </c>
-    </row>
-    <row r="263">
-      <c r="A263" t="inlineStr">
-        <is>
-          <t>SKWD</t>
-        </is>
-      </c>
-    </row>
-    <row r="264">
-      <c r="A264" t="inlineStr">
-        <is>
-          <t>SLDE</t>
-        </is>
-      </c>
-    </row>
-    <row r="265">
-      <c r="A265" t="inlineStr">
-        <is>
-          <t>SMPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="266">
-      <c r="A266" t="inlineStr">
-        <is>
-          <t>SPSC</t>
-        </is>
-      </c>
-    </row>
-    <row r="267">
-      <c r="A267" t="inlineStr">
-        <is>
           <t>SPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="268">
-      <c r="A268" t="inlineStr">
-        <is>
-          <t>TONT</t>
-        </is>
-      </c>
-    </row>
-    <row r="269">
-      <c r="A269" t="inlineStr">
-        <is>
-          <t>TRS</t>
-        </is>
-      </c>
-    </row>
-    <row r="270">
-      <c r="A270" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-    </row>
-    <row r="271">
-      <c r="A271" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
-    </row>
-    <row r="272">
-      <c r="A272" t="inlineStr">
-        <is>
-          <t>XZO</t>
-        </is>
-      </c>
-    </row>
-    <row r="273">
-      <c r="A273" t="inlineStr">
-        <is>
-          <t>YSWY</t>
-        </is>
-      </c>
-    </row>
-    <row r="274">
-      <c r="A274" t="inlineStr">
-        <is>
-          <t>ETS</t>
-        </is>
-      </c>
-    </row>
-    <row r="275">
-      <c r="A275" t="inlineStr">
-        <is>
-          <t>JRVR</t>
-        </is>
-      </c>
-    </row>
-    <row r="276">
-      <c r="A276" t="inlineStr">
-        <is>
-          <t>BMBL</t>
-        </is>
-      </c>
-    </row>
-    <row r="277">
-      <c r="A277" t="inlineStr">
-        <is>
-          <t>MXCT</t>
-        </is>
-      </c>
-    </row>
-    <row r="278">
-      <c r="A278" t="inlineStr">
-        <is>
-          <t>INDP</t>
-        </is>
-      </c>
-    </row>
-    <row r="279">
-      <c r="A279" t="inlineStr">
-        <is>
-          <t>HPK</t>
-        </is>
-      </c>
-    </row>
-    <row r="280">
-      <c r="A280" t="inlineStr">
-        <is>
-          <t>ORIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="281">
-      <c r="A281" t="inlineStr">
-        <is>
-          <t>BLMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="282">
-      <c r="A282" t="inlineStr">
-        <is>
-          <t>OPK</t>
-        </is>
-      </c>
-    </row>
-    <row r="283">
-      <c r="A283" t="inlineStr">
-        <is>
-          <t>SKYA</t>
-        </is>
-      </c>
-    </row>
-    <row r="284">
-      <c r="A284" t="inlineStr">
-        <is>
-          <t>MAZE</t>
-        </is>
-      </c>
-    </row>
-    <row r="285">
-      <c r="A285" t="inlineStr">
-        <is>
-          <t>ENTX</t>
-        </is>
-      </c>
-    </row>
-    <row r="286">
-      <c r="A286" t="inlineStr">
-        <is>
-          <t>ICG</t>
-        </is>
-      </c>
-    </row>
-    <row r="287">
-      <c r="A287" t="inlineStr">
-        <is>
-          <t>PTLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="288">
-      <c r="A288" t="inlineStr">
-        <is>
-          <t>KPLT</t>
-        </is>
-      </c>
-    </row>
-    <row r="289">
-      <c r="A289" t="inlineStr">
-        <is>
-          <t>SKIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="290">
-      <c r="A290" t="inlineStr">
-        <is>
-          <t>RTSN</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-25
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A247"/>
+  <dimension ref="A1:A246"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -811,14 +811,14 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>CBFV</t>
         </is>
       </c>
     </row>
@@ -832,7 +832,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
@@ -846,7 +846,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
@@ -860,7 +860,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>CCSI</t>
         </is>
       </c>
     </row>
@@ -874,7 +874,7 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
@@ -888,21 +888,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>DMAC</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>DMAC</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
@@ -916,21 +916,21 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
@@ -944,21 +944,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
@@ -972,14 +972,14 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CZFS</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
@@ -993,21 +993,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>FUNC</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>FUNC</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
@@ -1021,7 +1021,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
@@ -1035,7 +1035,7 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>DHCNL</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
@@ -1063,21 +1063,21 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
@@ -1091,14 +1091,14 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>ETS</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>ETS</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
@@ -1112,14 +1112,14 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
@@ -1133,7 +1133,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
@@ -1147,7 +1147,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>FORR</t>
         </is>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FORR</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
@@ -1175,7 +1175,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
@@ -1189,7 +1189,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
@@ -1203,28 +1203,28 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>IPXG</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>IPXG</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
@@ -1238,14 +1238,14 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1259,7 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
@@ -1273,21 +1273,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
@@ -1301,14 +1301,14 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>HYNE</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
@@ -1322,7 +1322,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
@@ -1336,7 +1336,7 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>III</t>
         </is>
       </c>
     </row>
@@ -1350,7 +1350,7 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
@@ -1364,14 +1364,14 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>MTLS</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>MTLS</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
@@ -1385,14 +1385,14 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
@@ -1406,14 +1406,14 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
@@ -1427,7 +1427,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
@@ -1441,7 +1441,7 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>MGYR</t>
         </is>
       </c>
     </row>
@@ -1455,7 +1455,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MGYR</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
@@ -1469,7 +1469,7 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
@@ -1483,7 +1483,7 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
@@ -1497,7 +1497,7 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>NATH</t>
         </is>
       </c>
     </row>
@@ -1511,7 +1511,7 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>NAUT</t>
         </is>
       </c>
     </row>
@@ -1525,7 +1525,7 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1539,7 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>NBTB</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
@@ -1553,7 +1553,7 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>NIQ</t>
         </is>
       </c>
     </row>
@@ -1567,7 +1567,7 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
@@ -1581,14 +1581,14 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>NSSC</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>NTRSO</t>
         </is>
       </c>
     </row>
@@ -1602,14 +1602,14 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
@@ -1623,14 +1623,14 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>OABI</t>
         </is>
       </c>
     </row>
@@ -1644,7 +1644,7 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
@@ -1658,7 +1658,7 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
@@ -1672,7 +1672,7 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>ORIC</t>
         </is>
       </c>
     </row>
@@ -1686,7 +1686,7 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
@@ -1700,7 +1700,7 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
@@ -1714,28 +1714,28 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>POWW</t>
         </is>
       </c>
     </row>
@@ -1749,14 +1749,14 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>PRDO</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>PRME</t>
         </is>
       </c>
     </row>
@@ -1770,14 +1770,14 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>PSIG</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>PSIG</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
@@ -1791,14 +1791,14 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>REAL</t>
         </is>
       </c>
     </row>
@@ -1812,210 +1812,210 @@
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>REF</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>REF</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>SBFG</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>SBFG</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>SWKHL</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>TACO</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>TACO</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>CAPS</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>CAPS</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>MNDY</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>DGICB</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>OPK</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>JRVR</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>KINS</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>ALGN</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>OMH</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>MTEX</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>DGICB</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>ALGN</t>
+          <t>AEYE</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>SVIAW</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>EVAX</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>MTEX</t>
+          <t>OMH</t>
         </is>
       </c>
     </row>
@@ -2029,84 +2029,84 @@
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>SLE</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>JRVR</t>
+          <t>OLED</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>SVIAW</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>SLE</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>GP</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
@@ -2120,28 +2120,21 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>GP</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>OPK</t>
+          <t>EVAX</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>PCTY</t>
-        </is>
-      </c>
-    </row>
-    <row r="247">
-      <c r="A247" t="inlineStr">
-        <is>
-          <t>SPT</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-26
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A246"/>
+  <dimension ref="A1:A390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,7 +426,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AGBK</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
@@ -440,1701 +440,2709 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BHST</t>
+          <t>RENT</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AQB</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>FNWD</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ADAMI</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BVC</t>
+          <t>AQB</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ASR</t>
+          <t>FORTY</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>AIIR</t>
+          <t>ADAMI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>ARXS</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AIXI</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>AFYA</t>
+          <t>BDTX</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>EJH</t>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>LFS</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>BHST</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AHG</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>BVC</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AMRO</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>GRFS</t>
+          <t>CLBT</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>CTSO</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PLBY</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>DORM</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>KWY</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>FELE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>AISP</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>FLX</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>ALGN</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>RGC</t>
+          <t>GRFS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>BETR</t>
+          <t>HLMN</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>PEPG</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>HONA</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>BMBL</t>
+          <t>AMAL</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>HTZ</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>TCMD</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>KLRA</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>AMRO</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>KXIN</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>BDCI</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>LIF</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>AMSF</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>NYAX</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>BOTJ</t>
+          <t>API</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>OMH</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>OSG</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>BRBI</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>PECO</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>ASND</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>PMA</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>PSMT</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>ATGL</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>COFS</t>
+          <t>PWRL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>AUDC</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>CPIX</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>CWST</t>
+          <t>SNWV</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>SOLS</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>BBSI</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>DIBS</t>
+          <t>STAA</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>DMAC</t>
+          <t>BCAL</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>BCPC</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>TREE</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>DRDB</t>
+          <t>BOLT</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>BOTJ</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>BSIN</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>BSRR</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>BSY</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>BUSE</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CZFS</t>
+          <t>BVS</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>BWFG</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>BWMN</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>FUNC</t>
+          <t>BZUN</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>CAC</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>GAING</t>
+          <t>CAI</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>DHCNL</t>
+          <t>CAPS</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>GAINI</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>GAINZ</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>CBU</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>CCBG</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>CCSI</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>ETS</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>HEPS</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>CHA</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>CHAD</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>CHCO</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>FORR</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>HUIZ</t>
+          <t>CIVB</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>CNOB</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>CRON</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IPXG</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>CTSH</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>JCSE</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>DMAC</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>HYNE</t>
+          <t>DMLP</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>DSGX</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>EBAY</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>MBRX</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>ELMT</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>MMTX</t>
+          <t>ENSG</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>MTLS</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>ESLA</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>ESLT</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>EVCM</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>NPAC</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>EXC</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>NWFL</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>EXYN</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>ONBPP</t>
+          <t>FBIZ</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>MGYR</t>
+          <t>FCBC</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>FISI</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>OTLY</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>FIVN</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>OXLCZ</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>NATH</t>
+          <t>FMBH</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>PAX</t>
+          <t>FMNB</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>NBTB</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>PICS</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>FSSL</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>PMTS</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>NIQ</t>
+          <t>FUNC</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>GABC</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>GAING</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>GAINI</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>GAINZ</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>PTLE</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>GEHC</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>REBN</t>
+          <t>GIBO</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>GIII</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>OABI</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>REVB</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>GP</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>HAFC</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>ORIC</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>RWAYI</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>HIFS</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>HOPE</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>HPK</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>TBCH</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>PRDO</t>
+          <t>IA</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>IBCP</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>TRAX</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>PSIG</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>IDXX</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>REF</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>IRLA</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>SBFG</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>IRTC</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>TACO</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>JCAP</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>JCSE</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>CAPS</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>JMSB</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>JOYY</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>MNDY</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>KIDS</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>OPK</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>JRVR</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>LFCR</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>ALGN</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>MTEX</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>DGICB</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>LMRI</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>LNT</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>WTW</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>MBRX</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>OMH</t>
+          <t>MCBS</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>BMGL</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>MGRC</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>MITK</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>SLE</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>MMSI</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>SVIAW</t>
+          <t>MTC</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>MTEX</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>MTLS</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>GP</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>EXYN</t>
+          <t>NCNO</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>EVAX</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
+          <t>NSIT</t>
+        </is>
+      </c>
+    </row>
+    <row r="247">
+      <c r="A247" t="inlineStr">
+        <is>
+          <t>NSSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="248">
+      <c r="A248" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="249">
+      <c r="A249" t="inlineStr">
+        <is>
+          <t>NTRSO</t>
+        </is>
+      </c>
+    </row>
+    <row r="250">
+      <c r="A250" t="inlineStr">
+        <is>
+          <t>NWBI</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>NWE</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>NWFL</t>
+        </is>
+      </c>
+    </row>
+    <row r="253">
+      <c r="A253" t="inlineStr">
+        <is>
+          <t>OCTV</t>
+        </is>
+      </c>
+    </row>
+    <row r="254">
+      <c r="A254" t="inlineStr">
+        <is>
+          <t>OLED</t>
+        </is>
+      </c>
+    </row>
+    <row r="255">
+      <c r="A255" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+    </row>
+    <row r="256">
+      <c r="A256" t="inlineStr">
+        <is>
+          <t>OPRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="257">
+      <c r="A257" t="inlineStr">
+        <is>
+          <t>OPRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="258">
+      <c r="A258" t="inlineStr">
+        <is>
+          <t>ORRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="259">
+      <c r="A259" t="inlineStr">
+        <is>
+          <t>OSPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="260">
+      <c r="A260" t="inlineStr">
+        <is>
+          <t>OYSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="261">
+      <c r="A261" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="262">
+      <c r="A262" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="263">
+      <c r="A263" t="inlineStr">
+        <is>
+          <t>PBFS</t>
+        </is>
+      </c>
+    </row>
+    <row r="264">
+      <c r="A264" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="265">
+      <c r="A265" t="inlineStr">
+        <is>
+          <t>PCRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="266">
+      <c r="A266" t="inlineStr">
+        <is>
+          <t>PFBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="267">
+      <c r="A267" t="inlineStr">
+        <is>
+          <t>PLBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="268">
+      <c r="A268" t="inlineStr">
+        <is>
+          <t>PLUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="269">
+      <c r="A269" t="inlineStr">
+        <is>
+          <t>PMTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="270">
+      <c r="A270" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
+    </row>
+    <row r="271">
+      <c r="A271" t="inlineStr">
+        <is>
+          <t>PNTG</t>
+        </is>
+      </c>
+    </row>
+    <row r="272">
+      <c r="A272" t="inlineStr">
+        <is>
+          <t>POM</t>
+        </is>
+      </c>
+    </row>
+    <row r="273">
+      <c r="A273" t="inlineStr">
+        <is>
+          <t>POWW</t>
+        </is>
+      </c>
+    </row>
+    <row r="274">
+      <c r="A274" t="inlineStr">
+        <is>
+          <t>PRCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="275">
+      <c r="A275" t="inlineStr">
+        <is>
+          <t>PRGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="276">
+      <c r="A276" t="inlineStr">
+        <is>
+          <t>QCRH</t>
+        </is>
+      </c>
+    </row>
+    <row r="277">
+      <c r="A277" t="inlineStr">
+        <is>
+          <t>QDEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="278">
+      <c r="A278" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="279">
+      <c r="A279" t="inlineStr">
+        <is>
+          <t>QNBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="280">
+      <c r="A280" t="inlineStr">
+        <is>
+          <t>RCBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="281">
+      <c r="A281" t="inlineStr">
+        <is>
+          <t>REF</t>
+        </is>
+      </c>
+    </row>
+    <row r="282">
+      <c r="A282" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+    </row>
+    <row r="283">
+      <c r="A283" t="inlineStr">
+        <is>
+          <t>RGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="284">
+      <c r="A284" t="inlineStr">
+        <is>
+          <t>RIGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="285">
+      <c r="A285" t="inlineStr">
+        <is>
+          <t>ROKU</t>
+        </is>
+      </c>
+    </row>
+    <row r="286">
+      <c r="A286" t="inlineStr">
+        <is>
+          <t>ROP</t>
+        </is>
+      </c>
+    </row>
+    <row r="287">
+      <c r="A287" t="inlineStr">
+        <is>
+          <t>RPD</t>
+        </is>
+      </c>
+    </row>
+    <row r="288">
+      <c r="A288" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="289">
+      <c r="A289" t="inlineStr">
+        <is>
+          <t>RUSHB</t>
+        </is>
+      </c>
+    </row>
+    <row r="290">
+      <c r="A290" t="inlineStr">
+        <is>
+          <t>RVSB</t>
+        </is>
+      </c>
+    </row>
+    <row r="291">
+      <c r="A291" t="inlineStr">
+        <is>
+          <t>RYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="292">
+      <c r="A292" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="293">
+      <c r="A293" t="inlineStr">
+        <is>
+          <t>SBCF</t>
+        </is>
+      </c>
+    </row>
+    <row r="294">
+      <c r="A294" t="inlineStr">
+        <is>
+          <t>SBFG</t>
+        </is>
+      </c>
+    </row>
+    <row r="295">
+      <c r="A295" t="inlineStr">
+        <is>
+          <t>SCSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="296">
+      <c r="A296" t="inlineStr">
+        <is>
+          <t>SEPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="297">
+      <c r="A297" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+    </row>
+    <row r="298">
+      <c r="A298" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="299">
+      <c r="A299" t="inlineStr">
+        <is>
+          <t>SGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="300">
+      <c r="A300" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+    </row>
+    <row r="301">
+      <c r="A301" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="302">
+      <c r="A302" t="inlineStr">
+        <is>
+          <t>SKYA</t>
+        </is>
+      </c>
+    </row>
+    <row r="303">
+      <c r="A303" t="inlineStr">
+        <is>
+          <t>SLDE</t>
+        </is>
+      </c>
+    </row>
+    <row r="304">
+      <c r="A304" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="305">
+      <c r="A305" t="inlineStr">
+        <is>
+          <t>SONO</t>
+        </is>
+      </c>
+    </row>
+    <row r="306">
+      <c r="A306" t="inlineStr">
+        <is>
+          <t>SPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="307">
+      <c r="A307" t="inlineStr">
+        <is>
+          <t>SRCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="308">
+      <c r="A308" t="inlineStr">
+        <is>
+          <t>SSNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="309">
+      <c r="A309" t="inlineStr">
+        <is>
+          <t>STBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="310">
+      <c r="A310" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="311">
+      <c r="A311" t="inlineStr">
+        <is>
+          <t>STLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="312">
+      <c r="A312" t="inlineStr">
+        <is>
+          <t>SUNB</t>
+        </is>
+      </c>
+    </row>
+    <row r="313">
+      <c r="A313" t="inlineStr">
+        <is>
+          <t>SWKHL</t>
+        </is>
+      </c>
+    </row>
+    <row r="314">
+      <c r="A314" t="inlineStr">
+        <is>
+          <t>SYNA</t>
+        </is>
+      </c>
+    </row>
+    <row r="315">
+      <c r="A315" t="inlineStr">
+        <is>
+          <t>SYRE</t>
+        </is>
+      </c>
+    </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>TACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>TCMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>TILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>TRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>TRS</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>WAFU</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>WLTH</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>WSBCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>YMAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>YSWY</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>OZK</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>PCTY</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>ACIW</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>OPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>XLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>INTA</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>ARHS</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>EFOR</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>AVTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>EMBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>TBCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>ASBH</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>BMGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>DOX</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>FTDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>MORN</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>APPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>ASRV</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>BIIB</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>MANH</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>HON</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>STFS</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>TRAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>EPSN</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>AGNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>FRSH</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>PBYI</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>POOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>HQY</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>NTWK</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>AMPL</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>CWST</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>GRDX</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>MNDY</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>NIQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>DOCU</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>CDLR</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>BL</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>AVAH</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>REVB</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>CDZI</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>DBX</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>SGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>BETR</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>RPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>INGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>FA</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>SLE</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
           <t>KINS</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>DGICB</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>BLKB</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>COO</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>BRCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>OTEX</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>JJSF</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>CINF</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>ICG</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>HCSG</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>CVBF</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>CDW</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-27
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A390"/>
+  <dimension ref="A1:A320"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,140 +426,140 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>AEYE</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABLV</t>
+          <t>ACT</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>RENT</t>
+          <t>ALGN</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>FNWD</t>
+          <t>ACU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACNB</t>
+          <t>AMSF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>AQB</t>
+          <t>JCSE</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>FORTY</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ADAMI</t>
+          <t>BGSI</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ARXS</t>
+          <t>KELYB</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BDTX</t>
+          <t>BMGL</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>POM</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>BHST</t>
+          <t>CARR</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BVC</t>
+          <t>CASH</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CLBT</t>
+          <t>CCB</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>AMAL</t>
         </is>
       </c>
     </row>
@@ -573,2576 +573,2086 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>DHCNI</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AMRO</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>FELE</t>
+          <t>EJH</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AISP</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>FLX</t>
+          <t>ELUT</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ALGN</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>GRFS</t>
+          <t>FLX</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>APPN</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>HLMN</t>
+          <t>IMCR</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HONA</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AMAL</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HTZ</t>
+          <t>KLRA</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KLRA</t>
+          <t>LIF</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AMRO</t>
+          <t>ARXS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>KXIN</t>
+          <t>NXPI</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>ASTL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>LIF</t>
+          <t>NYAX</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>OIO</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>NYAX</t>
+          <t>AUDC</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>OKYO</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>OMH</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>PWRL</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>AVBH</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>RSVR</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>BANR</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>PMA</t>
+          <t>SOLS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>PSMT</t>
+          <t>BCAL</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ATGL</t>
+          <t>STAA</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>BETR</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>TCBK</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PWRL</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>TREE</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>SBAC</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>VMRK</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SNWV</t>
+          <t>BOTJ</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BBSI</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>STAA</t>
+          <t>BSIN</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BCAL</t>
+          <t>BSRR</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BCPC</t>
+          <t>BSVN</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>TREE</t>
+          <t>BUSE</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BOLT</t>
+          <t>BVC</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BOTJ</t>
+          <t>BVS</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>BWFG</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>BWMN</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>CASS</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>BSIN</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>BSRR</t>
+          <t>CCID</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>BSY</t>
+          <t>CCSI</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BUSE</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BVS</t>
+          <t>CDW</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BWFG</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BWMN</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>CHDN</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>BZUN</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>CNXC</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>CRSR</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CAPS</t>
+          <t>CTKB</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>CTSH</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>CVLT</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CBU</t>
+          <t>CYRX</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CCBG</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>DOCU</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CHA</t>
+          <t>ERIC</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CHAD</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>EXE</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CIVB</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>EXYN</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>CNOB</t>
+          <t>FBIZ</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>FCBM</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>COFS</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CRON</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CRSR</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>FMBH</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>FRME</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>FSSL</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CZFS</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>FUNC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>FVNNU</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>GAINI</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>GCBC</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>DIBS</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>DMAC</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>DMLP</t>
+          <t>GRDX</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>GRFS</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>DSGX</t>
+          <t>GSBC</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>EBAY</t>
+          <t>GTM</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>HAFC</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>HBT</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>HCSG</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>ENSG</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>HON</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>ESLA</t>
+          <t>HOPE</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>EVCM</t>
+          <t>HWBK</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>EXC</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>EXYN</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>FBIZ</t>
+          <t>IMC</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>FCBC</t>
+          <t>IMKTA</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>FISI</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>IOVA</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>JBDI</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>FMBH</t>
+          <t>JOUT</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>FMNB</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>KELYA</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>KIDS</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>FRAF</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>KMRK</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>FSSL</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>FUNC</t>
+          <t>KRNT</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>GABC</t>
+          <t>KRRO</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>GAING</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>GAINI</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>GAINZ</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>LNT</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>LOGI</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>GEHC</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>MBWM</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>GP</t>
+          <t>MGRC</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>HAFC</t>
+          <t>MIDD</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>MLKN</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>MOBI</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>MQ</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>MTC</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>HIFS</t>
+          <t>MTLS</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>HOPE</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>HPK</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>NBBK</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>NECB</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>NMFCZ</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>HWKN</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>HYNE</t>
+          <t>NSSC</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>NTRSO</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>NWFL</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>OBT</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>OFIX</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>OPCH</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>OTAI</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>IRLA</t>
+          <t>PBYI</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>PDLB</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>PFIS</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>PFXNZ</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>PHAR</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>JCAP</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>JCSE</t>
+          <t>PLUS</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>PNFP</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>JMSB</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>JOYY</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>PRME</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>QCRH</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>QSI</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>RBB</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>LFCR</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>RDWR</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>RGS</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>LMRI</t>
+          <t>RILYG</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>ROKU</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>RPAY</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>RPC</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>MBRX</t>
+          <t>RRBI</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>MCBS</t>
+          <t>RVSB</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>MGRC</t>
+          <t>SAGT</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>MITK</t>
+          <t>SAIL</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>SBFG</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>MMSI</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>MTC</t>
+          <t>SFNC</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>MTEX</t>
+          <t>SGP</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>MTLS</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>SNFCA</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>NBTB</t>
+          <t>SPT</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>NCNO</t>
+          <t>SRCE</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>STBA</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>STRC</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>SUNB</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>SWIM</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>SYRE</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>TACT</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>TASK</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>NWFL</t>
+          <t>TCX</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>THFF</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>TILE</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>TOP</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>TOWN</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>TRAX</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>ORRF</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>OYSE</t>
+          <t>TRMD</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>TROO</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>TRS</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>PBFS</t>
+          <t>WCCB</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>WLTH</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>PCRX</t>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>PFBC</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>PLBC</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>POWW</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>PMTS</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>FIVN</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>POM</t>
+          <t>ESLA</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>FIBK</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>QCRH</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>ATGL</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>REF</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>SEPN</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>RGS</t>
+          <t>KXIN</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>CHMG</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>INVE</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>BBT</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>RUSHB</t>
+          <t>ELMT</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>OMH</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>SBCF</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>SBFG</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>SCSC</t>
+          <t>RENT</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>SEPN</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>TENB</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>SONO</t>
+          <t>OLED</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>SRCE</t>
+          <t>PLSE</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>SSNC</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>STBA</t>
+          <t>MGRT</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>STLD</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>STLN</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>SWKHL</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>IRTC</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>TACT</t>
+          <t>ORRF</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>TCMD</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>TILE</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>TRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="321">
-      <c r="A321" t="inlineStr">
-        <is>
-          <t>TRMB</t>
-        </is>
-      </c>
-    </row>
-    <row r="322">
-      <c r="A322" t="inlineStr">
-        <is>
-          <t>TRS</t>
-        </is>
-      </c>
-    </row>
-    <row r="323">
-      <c r="A323" t="inlineStr">
-        <is>
-          <t>TW</t>
-        </is>
-      </c>
-    </row>
-    <row r="324">
-      <c r="A324" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-    </row>
-    <row r="325">
-      <c r="A325" t="inlineStr">
-        <is>
-          <t>WAFU</t>
-        </is>
-      </c>
-    </row>
-    <row r="326">
-      <c r="A326" t="inlineStr">
-        <is>
-          <t>WLTH</t>
-        </is>
-      </c>
-    </row>
-    <row r="327">
-      <c r="A327" t="inlineStr">
-        <is>
-          <t>WSBCO</t>
-        </is>
-      </c>
-    </row>
-    <row r="328">
-      <c r="A328" t="inlineStr">
-        <is>
-          <t>YMAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="329">
-      <c r="A329" t="inlineStr">
-        <is>
-          <t>YSWY</t>
-        </is>
-      </c>
-    </row>
-    <row r="330">
-      <c r="A330" t="inlineStr">
-        <is>
-          <t>OZK</t>
-        </is>
-      </c>
-    </row>
-    <row r="331">
-      <c r="A331" t="inlineStr">
-        <is>
-          <t>PCTY</t>
-        </is>
-      </c>
-    </row>
-    <row r="332">
-      <c r="A332" t="inlineStr">
-        <is>
-          <t>ACIW</t>
-        </is>
-      </c>
-    </row>
-    <row r="333">
-      <c r="A333" t="inlineStr">
-        <is>
-          <t>OPK</t>
-        </is>
-      </c>
-    </row>
-    <row r="334">
-      <c r="A334" t="inlineStr">
-        <is>
-          <t>XLAB</t>
-        </is>
-      </c>
-    </row>
-    <row r="335">
-      <c r="A335" t="inlineStr">
-        <is>
-          <t>INTA</t>
-        </is>
-      </c>
-    </row>
-    <row r="336">
-      <c r="A336" t="inlineStr">
-        <is>
-          <t>ARHS</t>
-        </is>
-      </c>
-    </row>
-    <row r="337">
-      <c r="A337" t="inlineStr">
-        <is>
-          <t>EFOR</t>
-        </is>
-      </c>
-    </row>
-    <row r="338">
-      <c r="A338" t="inlineStr">
-        <is>
-          <t>AVTR</t>
-        </is>
-      </c>
-    </row>
-    <row r="339">
-      <c r="A339" t="inlineStr">
-        <is>
-          <t>EMBC</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>TBCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>ASBH</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
-        <is>
-          <t>BMGL</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="inlineStr">
-        <is>
-          <t>DOX</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>FTDR</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t>MORN</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>APPN</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>ASRV</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>BIIB</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>MANH</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>HON</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>STFS</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="inlineStr">
-        <is>
-          <t>TRAX</t>
-        </is>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" t="inlineStr">
-        <is>
-          <t>EPSN</t>
-        </is>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" t="inlineStr">
-        <is>
-          <t>AGNT</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" t="inlineStr">
-        <is>
-          <t>FRSH</t>
-        </is>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" t="inlineStr">
-        <is>
-          <t>PBYI</t>
-        </is>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" t="inlineStr">
-        <is>
-          <t>POOL</t>
-        </is>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" t="inlineStr">
-        <is>
-          <t>HQY</t>
-        </is>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" t="inlineStr">
-        <is>
-          <t>NTWK</t>
-        </is>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" t="inlineStr">
-        <is>
-          <t>AMPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" t="inlineStr">
-        <is>
-          <t>CWST</t>
-        </is>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" t="inlineStr">
-        <is>
-          <t>GRDX</t>
-        </is>
-      </c>
-    </row>
-    <row r="363">
-      <c r="A363" t="inlineStr">
-        <is>
-          <t>MNDY</t>
-        </is>
-      </c>
-    </row>
-    <row r="364">
-      <c r="A364" t="inlineStr">
-        <is>
-          <t>NIQ</t>
-        </is>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" t="inlineStr">
-        <is>
-          <t>DOCU</t>
-        </is>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" t="inlineStr">
-        <is>
-          <t>CDLR</t>
-        </is>
-      </c>
-    </row>
-    <row r="367">
-      <c r="A367" t="inlineStr">
-        <is>
-          <t>BL</t>
-        </is>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" t="inlineStr">
-        <is>
-          <t>AVAH</t>
-        </is>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" t="inlineStr">
-        <is>
-          <t>REVB</t>
-        </is>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" t="inlineStr">
-        <is>
-          <t>CDZI</t>
-        </is>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" t="inlineStr">
-        <is>
-          <t>DBX</t>
-        </is>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" t="inlineStr">
-        <is>
-          <t>SGHT</t>
-        </is>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" t="inlineStr">
-        <is>
-          <t>BETR</t>
-        </is>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="inlineStr">
-        <is>
-          <t>RPC</t>
-        </is>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" t="inlineStr">
-        <is>
-          <t>INGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="376">
-      <c r="A376" t="inlineStr">
-        <is>
-          <t>FA</t>
-        </is>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="inlineStr">
-        <is>
-          <t>SLE</t>
-        </is>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="inlineStr">
-        <is>
-          <t>KINS</t>
-        </is>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" t="inlineStr">
-        <is>
-          <t>DGICB</t>
-        </is>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="inlineStr">
-        <is>
-          <t>BLKB</t>
-        </is>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" t="inlineStr">
-        <is>
-          <t>COO</t>
-        </is>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" t="inlineStr">
-        <is>
-          <t>BRCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="inlineStr">
-        <is>
-          <t>OTEX</t>
-        </is>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" t="inlineStr">
-        <is>
-          <t>JJSF</t>
-        </is>
-      </c>
-    </row>
-    <row r="385">
-      <c r="A385" t="inlineStr">
-        <is>
-          <t>CINF</t>
-        </is>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" t="inlineStr">
-        <is>
-          <t>ICG</t>
-        </is>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" t="inlineStr">
-        <is>
-          <t>HCSG</t>
-        </is>
-      </c>
-    </row>
-    <row r="389">
-      <c r="A389" t="inlineStr">
-        <is>
-          <t>CVBF</t>
-        </is>
-      </c>
-    </row>
-    <row r="390">
-      <c r="A390" t="inlineStr">
-        <is>
-          <t>CDW</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-28
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A320"/>
+  <dimension ref="A1:A341"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,2233 +426,2380 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>AXIN</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALGN</t>
+          <t>BKYI</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>ALGN</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ACU</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>AMSF</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>JCSE</t>
+          <t>BANR</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>BGSI</t>
+          <t>ACT</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>KELYB</t>
+          <t>BBSI</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>ADAMI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>BMGL</t>
+          <t>CASH</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>POM</t>
+          <t>JVA</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CARR</t>
+          <t>CCB</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>KIDS</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>CIGI</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>CCB</t>
+          <t>PACB</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AMAL</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CTSO</t>
+          <t>CNDT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>POM</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>DHCNI</t>
+          <t>AEYE</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>AMRO</t>
+          <t>CTSO</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>EJH</t>
+          <t>PRME</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>ELUT</t>
+          <t>CVSA</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>SDHIU</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>FLX</t>
+          <t>AGIO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>APPN</t>
+          <t>DGNX</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IMCR</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>DHCNI</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>ELUT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>KLRA</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>FCCO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>LIF</t>
+          <t>ALRS</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>ARXS</t>
+          <t>FTW</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>AMAL</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ASTL</t>
+          <t>HLMN</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>NYAX</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>HONA</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>OIO</t>
+          <t>AMPL</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>JDZG</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>OKYO</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>KLTR</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>AOUT</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>KRMD</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>PWRL</t>
+          <t>API</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AVBH</t>
+          <t>LBRX</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>RSVR</t>
+          <t>AQB</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>LULU</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>BCAL</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>STAA</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>BETR</t>
+          <t>OIO</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>AROW</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>PCSA</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TREE</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>PEBO</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>BOTJ</t>
+          <t>PECO</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>ARXS</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>SNES</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>ASND</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>BSIN</t>
+          <t>SNY</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>BSRR</t>
+          <t>ASRV</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>TCMD</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>BUSE</t>
+          <t>ASTL</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>BVC</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>BVS</t>
+          <t>ATER</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>BWFG</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>BWMN</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>CASS</t>
+          <t>AVBH</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>CCID</t>
+          <t>AZTA</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>BBT</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>BDCI</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>BLLN</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>BLZR</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>BPRN</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>CNXC</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>CRSR</t>
+          <t>BSIN</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>CTKB</t>
+          <t>BSP</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>CTSH</t>
+          <t>BSRR</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>BWFG</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>CVLT</t>
+          <t>BWMN</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CZFS</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>CCBG</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>CCID</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>DOCU</t>
+          <t>CCSI</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>CHMG</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>CIVB</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>EXYN</t>
+          <t>CLBT</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>FBIZ</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FCBM</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>CPSS</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>CTKB</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>FMBH</t>
+          <t>CWST</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>CYRX</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>FRME</t>
+          <t>DAKT</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>FSSL</t>
+          <t>DBX</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>FUNC</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>FVNNU</t>
+          <t>DMAC</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>GAINI</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>GCBC</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>EFOR</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>ELMT</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>GRFS</t>
+          <t>EXEL</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>GSBC</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>GTM</t>
+          <t>FBNC</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>HAFC</t>
+          <t>FCAP</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>HBT</t>
+          <t>FCBM</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>FIVE</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>FIVN</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>HOPE</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>FMBH</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>HWBK</t>
+          <t>FMNB</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>HWKN</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>FROG</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>FSBC</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>FTRE</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>IMKTA</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>FVN</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>FVNNU</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>GRAL</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>IOVA</t>
+          <t>GSBC</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>JBDI</t>
+          <t>HAFC</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>JOUT</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>KELYA</t>
+          <t>HCSG</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>KINS</t>
+          <t>HMR</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>HON</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>HSTM</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>KRNT</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>KRRO</t>
+          <t>IA</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>IBEX</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>ICG</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>ILMN</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>LOGI</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>LSBK</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>INTA</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>MBWM</t>
+          <t>IRTC</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>MGRC</t>
+          <t>ISBA</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>MLKN</t>
+          <t>JJSF</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>MOBI</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>MQ</t>
+          <t>JMSB</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>MTC</t>
+          <t>JYD</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>MTLS</t>
+          <t>KARO</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>KELYA</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>KMRK</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>NBBK</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>NBTB</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>NECB</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>NMFCZ</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>KYIV</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>NTRSO</t>
+          <t>LEGN</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>NWFL</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>OBT</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>LMRI</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>MBWM</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>PBYI</t>
+          <t>MCBS</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>PDLB</t>
+          <t>MEDP</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>PFIS</t>
+          <t>MGPI</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>PFXNZ</t>
+          <t>MGRT</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>MOBI</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>MSBI</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>MWYN</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>NAUT</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>NBN</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>QCRH</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>QSI</t>
+          <t>NECB</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>RBB</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>NMIH</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>NRC</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>RGS</t>
+          <t>NTNX</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>RILYG</t>
+          <t>NTRA</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>ROKU</t>
+          <t>NTSK</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>OFIX</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>OM</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>RRBI</t>
+          <t>OMCL</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>RVSB</t>
+          <t>ONC</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>OPCH</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>OPRX</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>SAGT</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>SAIL</t>
+          <t>OTEX</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>SBFG</t>
+          <t>OVBC</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>PDLB</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>PHAR</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>PLSE</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>PNRG</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>SNFCA</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>POWW</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>SPT</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>SRCE</t>
+          <t>PRCH</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>STBA</t>
+          <t>PRCT</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>STRC</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>PRTH</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>PSIG</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>SYNA</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>QCRH</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>TACT</t>
+          <t>QDEL</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>TASK</t>
+          <t>QLYS</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>TCX</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>THFF</t>
+          <t>QSI</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>TILE</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>TOP</t>
+          <t>RDVT</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>TOWN</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>TRAX</t>
+          <t>RMBI</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>TRI</t>
+          <t>RPD</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>RRBI</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>RWAYI</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>TROO</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>TRS</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>WCCB</t>
+          <t>SEPN</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>WLTH</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>SGHT</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>SGMT</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>SGP</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>SHOE</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>SHPH</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>SIBN</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>ESLA</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>SPSC</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>SRZN</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>STAA</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>STAK</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>STRC</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>SUNB</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>SWIM</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>ATGL</t>
+          <t>SWKS</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>SWRD</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>SEPN</t>
+          <t>SYRE</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>KXIN</t>
+          <t>TECH</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>CHMG</t>
+          <t>TENB</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>TRAX</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>INVE</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>TRMD</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>TROO</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>OMH</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>VALU</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>WCCB</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>RENT</t>
+          <t>XZO</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>DIBS</t>
+          <t>YORW</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>BETR</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>XFOR</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>MGRC</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>CLAR</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>BMGL</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>SLN</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>RENT</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>SGRY</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MGRT</t>
+          <t>RDWR</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>ABVC</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>ESLA</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>TACT</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>SAIL</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>ORRF</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>NTWK</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>NWFL</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>ATGL</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>GIBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>DOO</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>CGNT</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>ESQ</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>CINF</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>NWE</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>KXIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>DIBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>TNDM</t>
+        </is>
+      </c>
+    </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>AMRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>CDZI</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>KRRO</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>GRDX</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>CBFV</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>RPRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>PYPD</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>ENGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>NSSC</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>IMC</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>SAGT</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>OLED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-29
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A341"/>
+  <dimension ref="A1:A505"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,2380 +426,3528 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>AXIN</t>
+          <t>BSBK</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>PCSA</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BKYI</t>
+          <t>ALGN</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALGN</t>
+          <t>ABLV</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>ASR</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ACNB</t>
+          <t>CEPO</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>ABSI</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>CLAR</t>
+          <t>BANR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>COAG</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>BBSI</t>
+          <t>ACGL</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>ADAMI</t>
+          <t>DHCNI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>BBSI</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>CCB</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>BCBP</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>FVNNU</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>CIGI</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>PACB</t>
+          <t>BGSI</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>MAYS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>CNDT</t>
+          <t>ACT</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>POM</t>
+          <t>BKU</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>ACU</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CTSO</t>
+          <t>BOTJ</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>NUWE</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CVSA</t>
+          <t>CARG</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>SDHIU</t>
+          <t>PTLE</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>AGIO</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>DGNX</t>
+          <t>CASH</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>DHCNI</t>
+          <t>AER</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>CHDN</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>ELUT</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>AEYE</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>FCCO</t>
+          <t>CIGI</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>ALRS</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>FTW</t>
+          <t>CLBT</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>AMAL</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>HLMN</t>
+          <t>COLL</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>HONA</t>
+          <t>COO</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>AMPL</t>
+          <t>ALMR</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>JDZG</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>DORM</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>KLTR</t>
+          <t>ALRS</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>AOUT</t>
+          <t>EVER</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>KRMD</t>
+          <t>AMAL</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>EXE</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>LBRX</t>
+          <t>AMCR</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>AQB</t>
+          <t>EXYN</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>LULU</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>FHB</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>FISV</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>OIO</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>AROW</t>
+          <t>FLWS</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>PCSA</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>GIII</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>PEBO</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>AQB</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>HLMN</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ARXS</t>
+          <t>ARHS</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SNES</t>
+          <t>HOPE</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>ARLP</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SNY</t>
+          <t>IDN</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ASRV</t>
+          <t>AROW</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>TCMD</t>
+          <t>IVA</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ASTL</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>JMSB</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ATER</t>
+          <t>ASND</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>JRVR</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>AVBH</t>
+          <t>KLRA</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AVPT</t>
+          <t>ASTL</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>KRMD</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>ATEC</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>BDCI</t>
+          <t>KXIN</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>LIF</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>BLLN</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>BLZR</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>BPRN</t>
+          <t>ATR</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>LWAY</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>BSIN</t>
+          <t>ATRC</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BSP</t>
+          <t>MVBF</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>BSRR</t>
+          <t>AUDC</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>BWFG</t>
+          <t>NXST</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BWMN</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>OSIS</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>PATK</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>AVBH</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>PECO</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>CCBG</t>
+          <t>AZ</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>CCID</t>
+          <t>PLAY</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>CCSI</t>
+          <t>AZN</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>PLUR</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>AZTA</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>PRPL</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>BANF</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>QNST</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>BBT</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>CHMG</t>
+          <t>RARE</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>CIVB</t>
+          <t>BETR</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>CLBT</t>
+          <t>RBB</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>COFS</t>
+          <t>BFST</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>RSVR</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>CPSS</t>
+          <t>BHRB</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>BLLN</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CTKB</t>
+          <t>SMBC</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>BMRC</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CWST</t>
+          <t>SNES</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CYRX</t>
+          <t>BOBS</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>DAKT</t>
+          <t>SYBT</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>DBX</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>TCBK</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>DHCNL</t>
+          <t>TCBS</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>DMAC</t>
+          <t>BRLT</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>DMRC</t>
+          <t>TOWN</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>BSET</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>EFOR</t>
+          <t>TREE</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>BSP</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>XFOR</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>BSVN</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>EXEL</t>
+          <t>XLAB</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>FBNC</t>
+          <t>YORW</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>FCAP</t>
+          <t>BVS</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>FCBM</t>
+          <t>BWFG</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>BWIN</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>CAC</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>CAI</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>FIVN</t>
+          <t>CARL</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>FMBH</t>
+          <t>CBK</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>FMNB</t>
+          <t>CBNK</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>FRAF</t>
+          <t>CBU</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>CCBG</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>FROG</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>FSBC</t>
+          <t>CD</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>FTRE</t>
+          <t>CDW</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>CDZI</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>FVN</t>
+          <t>CFBK</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>FVNNU</t>
+          <t>CFFI</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>CFR</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>GSBC</t>
+          <t>CHCO</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>HAFC</t>
+          <t>CHMG</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>CING</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>HLP</t>
+          <t>CIVB</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>HMR</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>CLMB</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>HSTM</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>COKE</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>COLB</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>IBEX</t>
+          <t>COLM</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>ICG</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>CTKB</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>ILMN</t>
+          <t>CV</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>CYPH</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>INTA</t>
+          <t>CZWI</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>DDOG</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>DGICA</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>ISBA</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>JJSF</t>
+          <t>DOO</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>JMSB</t>
+          <t>DTIL</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>JYD</t>
+          <t>DUKU</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>KARO</t>
+          <t>DYOR</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>KELYA</t>
+          <t>EBC</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>EFSI</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>EGBN</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>EGHT</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>ELMT</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>KYIV</t>
+          <t>EMBC</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>LEGN</t>
+          <t>ENVX</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>ERIC</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>ESLT</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>LMRI</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>LSBK</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>FBIZ</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>MBWM</t>
+          <t>FBLA</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>MCBS</t>
+          <t>FCAP</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>MEDP</t>
+          <t>FCBM</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>FCCO</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>MGRT</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>MOBI</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>MSBI</t>
+          <t>FFBC</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>MWYN</t>
+          <t>FGBI</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>FIBK</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>MYGN</t>
+          <t>FISI</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>NAUT</t>
+          <t>FITB</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>FIVE</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>NBTB</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>NECB</t>
+          <t>FMBH</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>FMNB</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>FNKO</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>NRC</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>FNWD</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>FRD</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>FRHC</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>NTSK</t>
+          <t>FRME</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>FRMEP</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>FSBC</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>OM</t>
+          <t>FSSL</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>FSV</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>OPCH</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>FUNC</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>FVN</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>OTEX</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>GDRX</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>GH</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>PDLB</t>
+          <t>GLBE</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>PHAR</t>
+          <t>GRAL</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>GSBC</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>PNRG</t>
+          <t>HAFC</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>HBIO</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>PPLC</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>PRCH</t>
+          <t>HBT</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>HCSG</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>HELE</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>PRTH</t>
+          <t>HIFS</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>PSIG</t>
+          <t>HON</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>HOWL</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>QCRH</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>HTFL</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>QSI</t>
+          <t>HWBK</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>RDVT</t>
+          <t>IA</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>IBCP</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>RMBI</t>
+          <t>ICLR</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>RPD</t>
+          <t>ICUI</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>RRBI</t>
+          <t>IDXX</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>RWAYI</t>
+          <t>IMC</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>SBAC</t>
+          <t>INDP</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>SEPN</t>
+          <t>INGN</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>SEZL</t>
+          <t>INTG</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>SGHT</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>SGMT</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>IRTC</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>SHOE</t>
+          <t>ISBA</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>SHPH</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>SIBN</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>SKYA</t>
+          <t>JJSF</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>SLDE</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>SPSC</t>
+          <t>JVA</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>SRZN</t>
+          <t>KARO</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>STAA</t>
+          <t>KIDS</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>STAK</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>STRC</t>
+          <t>KLTR</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>SUNB</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>SWIM</t>
+          <t>KNSA</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>SWKS</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>SWRD</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>SYRE</t>
+          <t>KRNT</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>TECH</t>
+          <t>KROS</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>TENB</t>
+          <t>KRRO</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>TLS</t>
+          <t>KRT</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>TRAX</t>
+          <t>KVHI</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>TRMB</t>
+          <t>KYIV</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>TRMD</t>
+          <t>LARK</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>TROO</t>
+          <t>LBRX</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>TW</t>
+          <t>LECO</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>UTHR</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>VALU</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>WCCB</t>
+          <t>LIND</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>XNCR</t>
+          <t>LIVN</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>XZO</t>
+          <t>LKFN</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>YORW</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>YSWY</t>
+          <t>LLYVA</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>BETR</t>
+          <t>LLYVK</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>XFOR</t>
+          <t>LMRI</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>MGRC</t>
+          <t>LNT</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>LOVE</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>LQDT</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>BMGL</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>SLN</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>RENT</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>SGRY</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>MBWM</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>MCBS</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>ABVC</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>ESLA</t>
+          <t>MGPI</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>TACT</t>
+          <t>MGRC</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>MGRT</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>SAIL</t>
+          <t>MIDD</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>BRCB</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>NTWK</t>
+          <t>MRSH</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>NWFL</t>
+          <t>MSBI</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>ATGL</t>
+          <t>MSEX</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>MTEX</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>DOO</t>
+          <t>MXCT</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>MYFW</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>MZTI</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>NAVN</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>NBBK</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>KXIN</t>
+          <t>NBN</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>DIBS</t>
+          <t>NBTX</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>TNDM</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>NECB</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>NICE</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>KRRO</t>
+          <t>NMIH</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>GRDX</t>
+          <t>NOVT</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>CBFV</t>
+          <t>NPAC</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>NRC</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>PYPD</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>NSIT</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>NSSC</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>SAGT</t>
+          <t>NTCT</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>NTGR</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>NTNX</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>NTRA</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>NUTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>NWBI</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>NXPI</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>OBT</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>OFIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>OFS</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>OMAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>OMCL</t>
+        </is>
+      </c>
+    </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>ONC</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>OPK</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>OPLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>OPRT</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>OPRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>ORKA</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>ORRF</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>OSG</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>OSPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>OSUR</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>OSW</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>OTAI</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>OTTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>OVBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>OVLY</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>OXLCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>OXLCZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>OZK</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>PAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>PACB</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>PAGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>PCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>PDLB</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>PDSB</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>PEBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>PFBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>PFIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>PGNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>PLBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>PLBY</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>PLGO</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>PLMR</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>PLSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>PLUS</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>PNFP</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>PNTG</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>PODD</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>POOL</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>POWW</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>PPLC</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>PRCT</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>PRME</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>PRVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>PSIG</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>PTON</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>QDEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>QLYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>QSI</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>RCBC</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>RCEL</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>REAL</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>REF</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>REGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>RELY</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>REYN</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>RGCO</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>RIGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>RLAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>RMBI</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>ROOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>RPAY</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>RPC</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>RRBI</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>RYZ</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>SBAC</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>SBFG</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>SCHL</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>SEPN</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>SEZL</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>SFNC</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>SFST</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>SGHT</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>SGP</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>SHOE</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>SHPH</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>SIBN</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>SIGI</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>SLAB</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>SNFCA</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>SNY</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>SOMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>SPFI</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>SPTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>SRCE</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>SRZN</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>SSTI</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>STAA</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>STBA</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>STLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>STRC</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>SUNB</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>SWIM</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>SWRD</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>TACO</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>TACT</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>TBCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>TCMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>TFSL</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>TGTX</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>THFF</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>TILE</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>TMCI</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>TNDM</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>TRAX</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>TRMB</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>TRMD</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>TW</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>UTHR</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>VSXY</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>WCCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>YMAT</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>ATGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>BMGL</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>GIBO</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>MEDP</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>BRCB</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>DIBS</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>MOBI</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>CERT</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>ENGS</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>MRVI</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>PNRG</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>PHAR</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>JLHL</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>BSIN</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>PYPD</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>BOLT</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>JYD</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>EFOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>NOVTU</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>ANIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>HLP</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>SAIC</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>RENT</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>RIBBU</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>ATER</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>SWKS</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>TLS</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>DGII</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>INM</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>HAS</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>MYGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>NTWK</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>SLN</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>AVPT</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>SAGT</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>RDWR</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>ITRI</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>LEGN</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>AMRX</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>RICK</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>GNSS</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>AIFA</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>BVC</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>BSRR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-30
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A505"/>
+  <dimension ref="A1:A414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,49 +426,49 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BSBK</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PCSA</t>
+          <t>ABCL</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALGN</t>
+          <t>BRKRP</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ABLV</t>
+          <t>AHRT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ASR</t>
+          <t>CHOW</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>CEPO</t>
+          <t>ABLV</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ABSI</t>
+          <t>HBNB</t>
         </is>
       </c>
     </row>
@@ -482,7 +482,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>COAG</t>
+          <t>FBIZ</t>
         </is>
       </c>
     </row>
@@ -496,3458 +496,2821 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>DHCNI</t>
+          <t>BBSI</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>BBSI</t>
+          <t>ACIC</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>FRAF</t>
+          <t>BCBP</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>BCBP</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>FVNNU</t>
+          <t>BGSI</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>ACNB</t>
+          <t>NSLRL</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>BGSI</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>MAYS</t>
+          <t>BOKF</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>ACT</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>BKU</t>
+          <t>ACU</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>ACU</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>BOTJ</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>NUWE</t>
+          <t>ADP</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>ADMA</t>
+          <t>CHDN</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CARG</t>
+          <t>SHOE</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>PTLE</t>
+          <t>ADPT</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>CLRO</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>CASH</t>
+          <t>ADSK</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>COLL</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>AER</t>
+          <t>TOMZ</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>STFS</t>
+          <t>AEP</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>AEYE</t>
+          <t>CRNT</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CIGI</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>CWST</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>CLBT</t>
+          <t>AGYS</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>DPZ</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>COLL</t>
+          <t>ALKS</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>EJH</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>COO</t>
+          <t>ALLT</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ALMR</t>
+          <t>ESTA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ALRM</t>
+          <t>ALRS</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>EVER</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>ALRS</t>
+          <t>AMGN</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>EVER</t>
+          <t>EXTR</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AMAL</t>
+          <t>AMRX</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>EXE</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>AMCR</t>
+          <t>APA</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>EXYN</t>
+          <t>IDN</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>API</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>FHB</t>
+          <t>IMCR</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>ANDG</t>
+          <t>INSG</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>FISV</t>
+          <t>AROW</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>KWY</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>FLWS</t>
+          <t>ARQT</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>LMAT</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>GIII</t>
+          <t>ARX</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>APOG</t>
+          <t>LWAY</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>AQB</t>
+          <t>ASBH</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>HLMN</t>
+          <t>MGEE</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ARHS</t>
+          <t>ASND</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>HOPE</t>
+          <t>NBIX</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ARLP</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>IDN</t>
+          <t>NBN</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>AROW</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>IVA</t>
+          <t>NXST</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>ATR</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>JMSB</t>
+          <t>NYAX</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>AUDC</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>JRVR</t>
+          <t>OFIX</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>ASO</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>KLRA</t>
+          <t>PATK</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>ASTL</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>KRMD</t>
+          <t>PAYX</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>ATEC</t>
+          <t>AVBH</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>KXIN</t>
+          <t>PECO</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>AWR</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>LIF</t>
+          <t>AXGN</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>PLUR</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>PRTA</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>ATR</t>
+          <t>BBCP</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>LWAY</t>
+          <t>QQQX</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>ATRC</t>
+          <t>RARE</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>MVBF</t>
+          <t>BFST</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>RDCM</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>BHRB</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>AVAH</t>
+          <t>BIIB</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>OSIS</t>
+          <t>SMBC</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>SOLS</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>AVBH</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>TCBK</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>AZ</t>
+          <t>BMGL</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>PLAY</t>
+          <t>TCX</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>AZN</t>
+          <t>BMRC</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>PLUR</t>
+          <t>VMRK</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>AZTA</t>
+          <t>BOOM</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>PRPL</t>
+          <t>YORW</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BANF</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>QNST</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BBT</t>
+          <t>BSBK</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>RARE</t>
+          <t>BSIN</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BETR</t>
+          <t>BSP</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>RBB</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>BFST</t>
+          <t>BVC</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>RSVR</t>
+          <t>BVFL</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BHRB</t>
+          <t>BWFG</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>BLLN</t>
+          <t>BZ</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SMBC</t>
+          <t>CARL</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>BMRC</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SNES</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>BOBS</t>
+          <t>CBK</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SYBT</t>
+          <t>CBU</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>CCEP</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>CCID</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>TCBS</t>
+          <t>CDLR</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>BRLT</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>TOWN</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>BSET</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>TREE</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>BSP</t>
+          <t>CHCO</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>XFOR</t>
+          <t>CHKP</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>BSVN</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>XLAB</t>
+          <t>CIGI</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>YORW</t>
+          <t>CING</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>BVS</t>
+          <t>CIVB</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>BWFG</t>
+          <t>CLGN</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>BWIN</t>
+          <t>CME</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>CAC</t>
+          <t>COAG</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>CAI</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>CARL</t>
+          <t>COLM</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>COST</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>CRAI</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CBK</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CBNK</t>
+          <t>CTAS</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CBRL</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CBU</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CCBG</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>CZWI</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>DCBO</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>CDW</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>CDZI</t>
+          <t>DGII</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>CFBK</t>
+          <t>DLTR</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>CFFI</t>
+          <t>DMAA</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>CFR</t>
+          <t>DMII</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>DORM</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>DSP</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>CHMG</t>
+          <t>DUKU</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>EFSC</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>CING</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>CIVB</t>
+          <t>ERIC</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>CLAR</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>CLMB</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>EVRG</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>COFS</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>COKE</t>
+          <t>EXLS</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>COLB</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>COLM</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>FANG</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>FBNC</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>CTKB</t>
+          <t>FCBM</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>CV</t>
+          <t>FCCO</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>CYPH</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>CZFS</t>
+          <t>FDBC</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>FGBI</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>CZWI</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>DDOG</t>
+          <t>FMAO</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>DGICA</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>DHCNL</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>FRBA</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>DOO</t>
+          <t>FRD</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>FRHC</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>DTIL</t>
+          <t>FRME</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>DUKU</t>
+          <t>FSBC</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>DYOR</t>
+          <t>FSSL</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>EBC</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>EDHL</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>EFSI</t>
+          <t>FUNC</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>EGBN</t>
+          <t>GAING</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>EGHT</t>
+          <t>GCBC</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>ELMT</t>
+          <t>GCL</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>EMBC</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>ENTX</t>
+          <t>GIBO</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>ENVX</t>
+          <t>GO</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>GRFS</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>GSAT</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>GSBC</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>ESLT</t>
+          <t>GTLB</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>HAFC</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>HALO</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>HAS</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>HBIO</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>FBIZ</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>FBLA</t>
+          <t>HELE</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>FCAP</t>
+          <t>HFWA</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>FCBM</t>
+          <t>HON</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>FCCO</t>
+          <t>HTHT</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>HWBK</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>FFBC</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>FGBI</t>
+          <t>ICFI</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>FIBK</t>
+          <t>IDXX</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>FISI</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>FITB</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>FIVE</t>
+          <t>INTU</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>FLYW</t>
+          <t>INVA</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>FMBH</t>
+          <t>IPAR</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>FMNB</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>FNKO</t>
+          <t>ISBA</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>ISRG</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>FNWD</t>
+          <t>ITRI</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>FRD</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>JJSF</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>FRME</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>FRMEP</t>
+          <t>JOUT</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>FSBC</t>
+          <t>JVA</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>FSSL</t>
+          <t>KARO</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>FSV</t>
+          <t>KELYA</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>FUNC</t>
+          <t>KMRK</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>FVN</t>
+          <t>KROS</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>LBRX</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>GDRX</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>GH</t>
+          <t>LEGH</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>GLBE</t>
+          <t>LEGN</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>GRAL</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>GSBC</t>
+          <t>LIFE</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>HAFC</t>
+          <t>LIN</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LKFN</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>HBIO</t>
+          <t>LKFT</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>LLYVA</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>HBT</t>
+          <t>LLYVK</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>HCSG</t>
+          <t>LMRI</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>HELE</t>
+          <t>LOVE</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>HIFS</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>LYEL</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>HOWL</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>HQY</t>
+          <t>MANH</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>HTFL</t>
+          <t>MAR</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>MASS</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>MAZE</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>HWBK</t>
+          <t>MBWM</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>HYNE</t>
+          <t>MCHX</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>IA</t>
+          <t>MGPI</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>IBCP</t>
+          <t>MGYR</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>ICLR</t>
+          <t>MICC</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>ICUI</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>IMC</t>
+          <t>MRSH</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>INDB</t>
+          <t>MRVI</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>INDP</t>
+          <t>MSBI</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>INGN</t>
+          <t>MSEX</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>INTG</t>
+          <t>MTEX</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>MYFW</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>MZTI</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>IRTC</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>ISBA</t>
+          <t>NBTX</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>NDAQ</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>NRC</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>JJSF</t>
+          <t>NRDS</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>NRIX</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>NTLA</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>KARO</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>KIDS</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>KINS</t>
+          <t>NWFL</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>KLTR</t>
+          <t>OBT</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>KMTS</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>KNSA</t>
+          <t>OIO</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>KOD</t>
+          <t>OLED</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>KPLT</t>
+          <t>OPK</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>KRNT</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>KROS</t>
+          <t>ORRF</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>KRRO</t>
+          <t>OSW</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>KRT</t>
+          <t>OVLY</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>KVHI</t>
+          <t>OZK</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>KYIV</t>
+          <t>PCB</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>LARK</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>LBRX</t>
+          <t>PDLB</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>LECO</t>
+          <t>PEBO</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>LFST</t>
+          <t>PFIS</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>PFXNZ</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>LIND</t>
+          <t>PGC</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>LIVN</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>LKFN</t>
+          <t>PLBC</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>LLYVA</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>PNFP</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>LMRI</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>LNT</t>
+          <t>PODD</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>LOVE</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>LQDT</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>LSBK</t>
+          <t>PTC</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>PTEN</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>MANE</t>
+          <t>PTLE</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>PTLO</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PWRL</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>PYPD</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>MBWM</t>
+          <t>QCRH</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>MCBS</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>RDWR</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>MGRC</t>
+          <t>REF</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>MGRT</t>
+          <t>RELL</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>MIDD</t>
+          <t>REYN</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>RIGL</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>MRSH</t>
+          <t>RMBI</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>MSBI</t>
+          <t>ROOT</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>MSEX</t>
+          <t>ROP</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>MTEX</t>
+          <t>RPRX</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>MXCT</t>
+          <t>RRBI</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>MYFW</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>SAFT</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>NAVN</t>
+          <t>SAGT</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>NBBK</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>NBTX</t>
+          <t>SCAG</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>NECB</t>
+          <t>SDGR</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>NICE</t>
+          <t>SFNC</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>NMIH</t>
+          <t>SGP</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>NOVT</t>
+          <t>SHPH</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>NPAC</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>NRC</t>
+          <t>SNES</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>SNFCA</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>SOMN</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>NSIT</t>
+          <t>SRCE</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>NSSC</t>
+          <t>SRPT</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>NTCT</t>
+          <t>SRZN</t>
         </is>
       </c>
     </row>
     <row r="340">
       <c r="A340" t="inlineStr">
         <is>
-          <t>NTGR</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
     <row r="341">
       <c r="A341" t="inlineStr">
         <is>
-          <t>NTNX</t>
+          <t>SYRE</t>
         </is>
       </c>
     </row>
     <row r="342">
       <c r="A342" t="inlineStr">
         <is>
-          <t>NTRA</t>
+          <t>TACT</t>
         </is>
       </c>
     </row>
     <row r="343">
       <c r="A343" t="inlineStr">
         <is>
-          <t>NUTX</t>
+          <t>TCMD</t>
         </is>
       </c>
     </row>
     <row r="344">
       <c r="A344" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>TGTX</t>
         </is>
       </c>
     </row>
     <row r="345">
       <c r="A345" t="inlineStr">
         <is>
-          <t>NXPI</t>
+          <t>THFF</t>
         </is>
       </c>
     </row>
     <row r="346">
       <c r="A346" t="inlineStr">
         <is>
-          <t>OBT</t>
+          <t>TILE</t>
         </is>
       </c>
     </row>
     <row r="347">
       <c r="A347" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="348">
       <c r="A348" t="inlineStr">
         <is>
-          <t>OFS</t>
+          <t>TRI</t>
         </is>
       </c>
     </row>
     <row r="349">
       <c r="A349" t="inlineStr">
         <is>
-          <t>OMAB</t>
+          <t>TRMB</t>
         </is>
       </c>
     </row>
     <row r="350">
       <c r="A350" t="inlineStr">
         <is>
-          <t>OMCL</t>
+          <t>TW</t>
         </is>
       </c>
     </row>
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>ONC</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="352">
       <c r="A352" t="inlineStr">
         <is>
-          <t>OPK</t>
+          <t>VIR</t>
         </is>
       </c>
     </row>
     <row r="353">
       <c r="A353" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>WCCB</t>
         </is>
       </c>
     </row>
     <row r="354">
       <c r="A354" t="inlineStr">
         <is>
-          <t>OPRT</t>
+          <t>WHK</t>
         </is>
       </c>
     </row>
     <row r="355">
       <c r="A355" t="inlineStr">
         <is>
-          <t>OPRX</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
     <row r="356">
       <c r="A356" t="inlineStr">
         <is>
-          <t>ORKA</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="357">
       <c r="A357" t="inlineStr">
         <is>
-          <t>ORRF</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="358">
       <c r="A358" t="inlineStr">
         <is>
-          <t>OSG</t>
+          <t>EFOI</t>
         </is>
       </c>
     </row>
     <row r="359">
       <c r="A359" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>STAA</t>
         </is>
       </c>
     </row>
     <row r="360">
       <c r="A360" t="inlineStr">
         <is>
-          <t>OSUR</t>
+          <t>BETR</t>
         </is>
       </c>
     </row>
     <row r="361">
       <c r="A361" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="362">
       <c r="A362" t="inlineStr">
         <is>
-          <t>OTAI</t>
+          <t>RIBBU</t>
         </is>
       </c>
     </row>
     <row r="363">
       <c r="A363" t="inlineStr">
         <is>
-          <t>OTTR</t>
+          <t>FIVE</t>
         </is>
       </c>
     </row>
     <row r="364">
       <c r="A364" t="inlineStr">
         <is>
-          <t>OVBC</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="365">
       <c r="A365" t="inlineStr">
         <is>
-          <t>OVLY</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="366">
       <c r="A366" t="inlineStr">
         <is>
-          <t>OXLCO</t>
+          <t>GNSS</t>
         </is>
       </c>
     </row>
     <row r="367">
       <c r="A367" t="inlineStr">
         <is>
-          <t>OXLCZ</t>
+          <t>SWIM</t>
         </is>
       </c>
     </row>
     <row r="368">
       <c r="A368" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="369">
       <c r="A369" t="inlineStr">
         <is>
-          <t>PAA</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
         <is>
-          <t>PACB</t>
+          <t>DOO</t>
         </is>
       </c>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
         <is>
-          <t>PAGP</t>
+          <t>APOG</t>
         </is>
       </c>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>ATEX</t>
         </is>
       </c>
     </row>
     <row r="373">
       <c r="A373" t="inlineStr">
         <is>
-          <t>PDLB</t>
+          <t>SGRY</t>
         </is>
       </c>
     </row>
     <row r="374">
       <c r="A374" t="inlineStr">
         <is>
-          <t>PDSB</t>
+          <t>PRPL</t>
         </is>
       </c>
     </row>
     <row r="375">
       <c r="A375" t="inlineStr">
         <is>
-          <t>PEBO</t>
+          <t>ORKA</t>
         </is>
       </c>
     </row>
     <row r="376">
       <c r="A376" t="inlineStr">
         <is>
-          <t>PFBC</t>
+          <t>IBG</t>
         </is>
       </c>
     </row>
     <row r="377">
       <c r="A377" t="inlineStr">
         <is>
-          <t>PFIS</t>
+          <t>TMCI</t>
         </is>
       </c>
     </row>
     <row r="378">
       <c r="A378" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>ATGL</t>
         </is>
       </c>
     </row>
     <row r="379">
       <c r="A379" t="inlineStr">
         <is>
-          <t>PLBC</t>
+          <t>ICON</t>
         </is>
       </c>
     </row>
     <row r="380">
       <c r="A380" t="inlineStr">
         <is>
-          <t>PLBY</t>
+          <t>GLSI</t>
         </is>
       </c>
     </row>
     <row r="381">
       <c r="A381" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>CTKB</t>
         </is>
       </c>
     </row>
     <row r="382">
       <c r="A382" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>LUNG</t>
         </is>
       </c>
     </row>
     <row r="383">
       <c r="A383" t="inlineStr">
         <is>
-          <t>PLSE</t>
+          <t>KRRO</t>
         </is>
       </c>
     </row>
     <row r="384">
       <c r="A384" t="inlineStr">
         <is>
-          <t>PLUS</t>
+          <t>CHSN</t>
         </is>
       </c>
     </row>
     <row r="385">
       <c r="A385" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>LVO</t>
         </is>
       </c>
     </row>
     <row r="386">
       <c r="A386" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>SGHT</t>
         </is>
       </c>
     </row>
     <row r="387">
       <c r="A387" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>REPL</t>
         </is>
       </c>
     </row>
     <row r="388">
       <c r="A388" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>AVPT</t>
         </is>
       </c>
     </row>
     <row r="389">
       <c r="A389" t="inlineStr">
         <is>
-          <t>POWW</t>
+          <t>KXIN</t>
         </is>
       </c>
     </row>
     <row r="390">
       <c r="A390" t="inlineStr">
         <is>
-          <t>PPLC</t>
+          <t>ATER</t>
         </is>
       </c>
     </row>
     <row r="391">
       <c r="A391" t="inlineStr">
         <is>
-          <t>PRCT</t>
+          <t>PHAR</t>
         </is>
       </c>
     </row>
     <row r="392">
       <c r="A392" t="inlineStr">
         <is>
-          <t>PRME</t>
+          <t>ALRM</t>
         </is>
       </c>
     </row>
     <row r="393">
       <c r="A393" t="inlineStr">
         <is>
-          <t>PRVA</t>
+          <t>TRMD</t>
         </is>
       </c>
     </row>
     <row r="394">
       <c r="A394" t="inlineStr">
         <is>
-          <t>PSIG</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="395">
       <c r="A395" t="inlineStr">
         <is>
-          <t>PTON</t>
+          <t>RJET</t>
         </is>
       </c>
     </row>
     <row r="396">
       <c r="A396" t="inlineStr">
         <is>
-          <t>QDEL</t>
+          <t>KVHI</t>
         </is>
       </c>
     </row>
     <row r="397">
       <c r="A397" t="inlineStr">
         <is>
-          <t>QLYS</t>
+          <t>PNRG</t>
         </is>
       </c>
     </row>
     <row r="398">
       <c r="A398" t="inlineStr">
         <is>
-          <t>QSI</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="399">
       <c r="A399" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>SEPN</t>
         </is>
       </c>
     </row>
     <row r="400">
       <c r="A400" t="inlineStr">
         <is>
-          <t>RCEL</t>
+          <t>MLTX</t>
         </is>
       </c>
     </row>
     <row r="401">
       <c r="A401" t="inlineStr">
         <is>
-          <t>REAL</t>
+          <t>CHMG</t>
         </is>
       </c>
     </row>
     <row r="402">
       <c r="A402" t="inlineStr">
         <is>
-          <t>REF</t>
+          <t>IMC</t>
         </is>
       </c>
     </row>
     <row r="403">
       <c r="A403" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="404">
       <c r="A404" t="inlineStr">
         <is>
-          <t>RELY</t>
+          <t>RCEL</t>
         </is>
       </c>
     </row>
     <row r="405">
       <c r="A405" t="inlineStr">
         <is>
-          <t>REYN</t>
+          <t>MOBI</t>
         </is>
       </c>
     </row>
     <row r="406">
       <c r="A406" t="inlineStr">
         <is>
-          <t>RGCO</t>
+          <t>LFST</t>
         </is>
       </c>
     </row>
     <row r="407">
       <c r="A407" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>ADMA</t>
         </is>
       </c>
     </row>
     <row r="408">
       <c r="A408" t="inlineStr">
         <is>
-          <t>RLAY</t>
+          <t>FFTT</t>
         </is>
       </c>
     </row>
     <row r="409">
       <c r="A409" t="inlineStr">
         <is>
-          <t>RMBI</t>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
     <row r="410">
       <c r="A410" t="inlineStr">
         <is>
-          <t>ROOT</t>
+          <t>JLHL</t>
         </is>
       </c>
     </row>
     <row r="411">
       <c r="A411" t="inlineStr">
         <is>
-          <t>RPAY</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="412">
       <c r="A412" t="inlineStr">
         <is>
-          <t>RPC</t>
+          <t>MYGN</t>
         </is>
       </c>
     </row>
     <row r="413">
       <c r="A413" t="inlineStr">
         <is>
-          <t>RRBI</t>
+          <t>MANE</t>
         </is>
       </c>
     </row>
     <row r="414">
       <c r="A414" t="inlineStr">
         <is>
-          <t>RYZ</t>
-        </is>
-      </c>
-    </row>
-    <row r="415">
-      <c r="A415" t="inlineStr">
-        <is>
-          <t>SBAC</t>
-        </is>
-      </c>
-    </row>
-    <row r="416">
-      <c r="A416" t="inlineStr">
-        <is>
-          <t>SBFG</t>
-        </is>
-      </c>
-    </row>
-    <row r="417">
-      <c r="A417" t="inlineStr">
-        <is>
-          <t>SCHL</t>
-        </is>
-      </c>
-    </row>
-    <row r="418">
-      <c r="A418" t="inlineStr">
-        <is>
-          <t>SEPN</t>
-        </is>
-      </c>
-    </row>
-    <row r="419">
-      <c r="A419" t="inlineStr">
-        <is>
-          <t>SEZL</t>
-        </is>
-      </c>
-    </row>
-    <row r="420">
-      <c r="A420" t="inlineStr">
-        <is>
-          <t>SFNC</t>
-        </is>
-      </c>
-    </row>
-    <row r="421">
-      <c r="A421" t="inlineStr">
-        <is>
-          <t>SFST</t>
-        </is>
-      </c>
-    </row>
-    <row r="422">
-      <c r="A422" t="inlineStr">
-        <is>
-          <t>SGHT</t>
-        </is>
-      </c>
-    </row>
-    <row r="423">
-      <c r="A423" t="inlineStr">
-        <is>
-          <t>SGP</t>
-        </is>
-      </c>
-    </row>
-    <row r="424">
-      <c r="A424" t="inlineStr">
-        <is>
-          <t>SHOE</t>
-        </is>
-      </c>
-    </row>
-    <row r="425">
-      <c r="A425" t="inlineStr">
-        <is>
-          <t>SHPH</t>
-        </is>
-      </c>
-    </row>
-    <row r="426">
-      <c r="A426" t="inlineStr">
-        <is>
-          <t>SIBN</t>
-        </is>
-      </c>
-    </row>
-    <row r="427">
-      <c r="A427" t="inlineStr">
-        <is>
-          <t>SIGI</t>
-        </is>
-      </c>
-    </row>
-    <row r="428">
-      <c r="A428" t="inlineStr">
-        <is>
-          <t>SLAB</t>
-        </is>
-      </c>
-    </row>
-    <row r="429">
-      <c r="A429" t="inlineStr">
-        <is>
-          <t>SNFCA</t>
-        </is>
-      </c>
-    </row>
-    <row r="430">
-      <c r="A430" t="inlineStr">
-        <is>
-          <t>SNY</t>
-        </is>
-      </c>
-    </row>
-    <row r="431">
-      <c r="A431" t="inlineStr">
-        <is>
-          <t>SOMN</t>
-        </is>
-      </c>
-    </row>
-    <row r="432">
-      <c r="A432" t="inlineStr">
-        <is>
-          <t>SPFI</t>
-        </is>
-      </c>
-    </row>
-    <row r="433">
-      <c r="A433" t="inlineStr">
-        <is>
-          <t>SPTX</t>
-        </is>
-      </c>
-    </row>
-    <row r="434">
-      <c r="A434" t="inlineStr">
-        <is>
-          <t>SRCE</t>
-        </is>
-      </c>
-    </row>
-    <row r="435">
-      <c r="A435" t="inlineStr">
-        <is>
-          <t>SRZN</t>
-        </is>
-      </c>
-    </row>
-    <row r="436">
-      <c r="A436" t="inlineStr">
-        <is>
-          <t>SSTI</t>
-        </is>
-      </c>
-    </row>
-    <row r="437">
-      <c r="A437" t="inlineStr">
-        <is>
-          <t>STAA</t>
-        </is>
-      </c>
-    </row>
-    <row r="438">
-      <c r="A438" t="inlineStr">
-        <is>
-          <t>STBA</t>
-        </is>
-      </c>
-    </row>
-    <row r="439">
-      <c r="A439" t="inlineStr">
-        <is>
-          <t>STLD</t>
-        </is>
-      </c>
-    </row>
-    <row r="440">
-      <c r="A440" t="inlineStr">
-        <is>
-          <t>STRC</t>
-        </is>
-      </c>
-    </row>
-    <row r="441">
-      <c r="A441" t="inlineStr">
-        <is>
-          <t>SUNB</t>
-        </is>
-      </c>
-    </row>
-    <row r="442">
-      <c r="A442" t="inlineStr">
-        <is>
-          <t>SWIM</t>
-        </is>
-      </c>
-    </row>
-    <row r="443">
-      <c r="A443" t="inlineStr">
-        <is>
-          <t>SWRD</t>
-        </is>
-      </c>
-    </row>
-    <row r="444">
-      <c r="A444" t="inlineStr">
-        <is>
-          <t>TACO</t>
-        </is>
-      </c>
-    </row>
-    <row r="445">
-      <c r="A445" t="inlineStr">
-        <is>
-          <t>TACT</t>
-        </is>
-      </c>
-    </row>
-    <row r="446">
-      <c r="A446" t="inlineStr">
-        <is>
-          <t>TBCH</t>
-        </is>
-      </c>
-    </row>
-    <row r="447">
-      <c r="A447" t="inlineStr">
-        <is>
-          <t>TCMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="448">
-      <c r="A448" t="inlineStr">
-        <is>
-          <t>TFSL</t>
-        </is>
-      </c>
-    </row>
-    <row r="449">
-      <c r="A449" t="inlineStr">
-        <is>
-          <t>TGTX</t>
-        </is>
-      </c>
-    </row>
-    <row r="450">
-      <c r="A450" t="inlineStr">
-        <is>
-          <t>THFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="451">
-      <c r="A451" t="inlineStr">
-        <is>
-          <t>TILE</t>
-        </is>
-      </c>
-    </row>
-    <row r="452">
-      <c r="A452" t="inlineStr">
-        <is>
-          <t>TMCI</t>
-        </is>
-      </c>
-    </row>
-    <row r="453">
-      <c r="A453" t="inlineStr">
-        <is>
-          <t>TNDM</t>
-        </is>
-      </c>
-    </row>
-    <row r="454">
-      <c r="A454" t="inlineStr">
-        <is>
-          <t>TRAX</t>
-        </is>
-      </c>
-    </row>
-    <row r="455">
-      <c r="A455" t="inlineStr">
-        <is>
-          <t>TRMB</t>
-        </is>
-      </c>
-    </row>
-    <row r="456">
-      <c r="A456" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="457">
-      <c r="A457" t="inlineStr">
-        <is>
-          <t>TW</t>
-        </is>
-      </c>
-    </row>
-    <row r="458">
-      <c r="A458" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-    </row>
-    <row r="459">
-      <c r="A459" t="inlineStr">
-        <is>
-          <t>VSXY</t>
-        </is>
-      </c>
-    </row>
-    <row r="460">
-      <c r="A460" t="inlineStr">
-        <is>
-          <t>WCCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="461">
-      <c r="A461" t="inlineStr">
-        <is>
-          <t>YMAT</t>
-        </is>
-      </c>
-    </row>
-    <row r="462">
-      <c r="A462" t="inlineStr">
-        <is>
-          <t>ATGL</t>
-        </is>
-      </c>
-    </row>
-    <row r="463">
-      <c r="A463" t="inlineStr">
-        <is>
-          <t>BMGL</t>
-        </is>
-      </c>
-    </row>
-    <row r="464">
-      <c r="A464" t="inlineStr">
-        <is>
-          <t>GIBO</t>
-        </is>
-      </c>
-    </row>
-    <row r="465">
-      <c r="A465" t="inlineStr">
-        <is>
-          <t>MEDP</t>
-        </is>
-      </c>
-    </row>
-    <row r="466">
-      <c r="A466" t="inlineStr">
-        <is>
-          <t>BRCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="467">
-      <c r="A467" t="inlineStr">
-        <is>
-          <t>DIBS</t>
-        </is>
-      </c>
-    </row>
-    <row r="468">
-      <c r="A468" t="inlineStr">
-        <is>
-          <t>MOBI</t>
-        </is>
-      </c>
-    </row>
-    <row r="469">
-      <c r="A469" t="inlineStr">
-        <is>
-          <t>CERT</t>
-        </is>
-      </c>
-    </row>
-    <row r="470">
-      <c r="A470" t="inlineStr">
-        <is>
-          <t>ENGS</t>
-        </is>
-      </c>
-    </row>
-    <row r="471">
-      <c r="A471" t="inlineStr">
-        <is>
-          <t>MRVI</t>
-        </is>
-      </c>
-    </row>
-    <row r="472">
-      <c r="A472" t="inlineStr">
-        <is>
-          <t>PNRG</t>
-        </is>
-      </c>
-    </row>
-    <row r="473">
-      <c r="A473" t="inlineStr">
-        <is>
-          <t>PHAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="474">
-      <c r="A474" t="inlineStr">
-        <is>
-          <t>JLHL</t>
-        </is>
-      </c>
-    </row>
-    <row r="475">
-      <c r="A475" t="inlineStr">
-        <is>
-          <t>BSIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="476">
-      <c r="A476" t="inlineStr">
-        <is>
-          <t>PYPD</t>
-        </is>
-      </c>
-    </row>
-    <row r="477">
-      <c r="A477" t="inlineStr">
-        <is>
-          <t>BOLT</t>
-        </is>
-      </c>
-    </row>
-    <row r="478">
-      <c r="A478" t="inlineStr">
-        <is>
-          <t>JYD</t>
-        </is>
-      </c>
-    </row>
-    <row r="479">
-      <c r="A479" t="inlineStr">
-        <is>
-          <t>EFOI</t>
-        </is>
-      </c>
-    </row>
-    <row r="480">
-      <c r="A480" t="inlineStr">
-        <is>
-          <t>NOVTU</t>
-        </is>
-      </c>
-    </row>
-    <row r="481">
-      <c r="A481" t="inlineStr">
-        <is>
-          <t>ANIX</t>
-        </is>
-      </c>
-    </row>
-    <row r="482">
-      <c r="A482" t="inlineStr">
-        <is>
-          <t>HLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="483">
-      <c r="A483" t="inlineStr">
-        <is>
-          <t>SAIC</t>
-        </is>
-      </c>
-    </row>
-    <row r="484">
-      <c r="A484" t="inlineStr">
-        <is>
-          <t>RENT</t>
-        </is>
-      </c>
-    </row>
-    <row r="485">
-      <c r="A485" t="inlineStr">
-        <is>
-          <t>RIBBU</t>
-        </is>
-      </c>
-    </row>
-    <row r="486">
-      <c r="A486" t="inlineStr">
-        <is>
-          <t>ATER</t>
-        </is>
-      </c>
-    </row>
-    <row r="487">
-      <c r="A487" t="inlineStr">
-        <is>
-          <t>SWKS</t>
-        </is>
-      </c>
-    </row>
-    <row r="488">
-      <c r="A488" t="inlineStr">
-        <is>
-          <t>TLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="489">
-      <c r="A489" t="inlineStr">
-        <is>
-          <t>DGII</t>
-        </is>
-      </c>
-    </row>
-    <row r="490">
-      <c r="A490" t="inlineStr">
-        <is>
-          <t>INM</t>
-        </is>
-      </c>
-    </row>
-    <row r="491">
-      <c r="A491" t="inlineStr">
-        <is>
-          <t>HAS</t>
-        </is>
-      </c>
-    </row>
-    <row r="492">
-      <c r="A492" t="inlineStr">
-        <is>
-          <t>MYGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="493">
-      <c r="A493" t="inlineStr">
-        <is>
-          <t>NTWK</t>
-        </is>
-      </c>
-    </row>
-    <row r="494">
-      <c r="A494" t="inlineStr">
-        <is>
           <t>SLN</t>
-        </is>
-      </c>
-    </row>
-    <row r="495">
-      <c r="A495" t="inlineStr">
-        <is>
-          <t>AVPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="496">
-      <c r="A496" t="inlineStr">
-        <is>
-          <t>SAGT</t>
-        </is>
-      </c>
-    </row>
-    <row r="497">
-      <c r="A497" t="inlineStr">
-        <is>
-          <t>RDWR</t>
-        </is>
-      </c>
-    </row>
-    <row r="498">
-      <c r="A498" t="inlineStr">
-        <is>
-          <t>ITRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="499">
-      <c r="A499" t="inlineStr">
-        <is>
-          <t>LEGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="500">
-      <c r="A500" t="inlineStr">
-        <is>
-          <t>AMRX</t>
-        </is>
-      </c>
-    </row>
-    <row r="501">
-      <c r="A501" t="inlineStr">
-        <is>
-          <t>RICK</t>
-        </is>
-      </c>
-    </row>
-    <row r="502">
-      <c r="A502" t="inlineStr">
-        <is>
-          <t>GNSS</t>
-        </is>
-      </c>
-    </row>
-    <row r="503">
-      <c r="A503" t="inlineStr">
-        <is>
-          <t>AIFA</t>
-        </is>
-      </c>
-    </row>
-    <row r="504">
-      <c r="A504" t="inlineStr">
-        <is>
-          <t>BVC</t>
-        </is>
-      </c>
-    </row>
-    <row r="505">
-      <c r="A505" t="inlineStr">
-        <is>
-          <t>BSRR</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Momentum scan results 2026-10-31
</commit_message>
<xml_diff>
--- a/results/momentum_failcodes_latest.xlsx
+++ b/results/momentum_failcodes_latest.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A414"/>
+  <dimension ref="A1:A339"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,385 +426,385 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CDNA</t>
+          <t>ACIW</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ABCL</t>
+          <t>AHRT</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>BRKRP</t>
+          <t>BBSI</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>AHRT</t>
+          <t>ABLV</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>CHOW</t>
+          <t>ACU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ABLV</t>
+          <t>BANR</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>HBNB</t>
+          <t>BOKF</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>BANR</t>
+          <t>AFRI</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>FBIZ</t>
+          <t>BCBP</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>ACGL</t>
+          <t>CLRO</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>BBSI</t>
+          <t>ACNB</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>GDYN</t>
+          <t>BGSI</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ACIC</t>
+          <t>CRNT</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>BCBP</t>
+          <t>ANIK</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>MEOH</t>
+          <t>BRKRP</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>ACIW</t>
+          <t>CWST</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>BGSI</t>
+          <t>CASY</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>NSLRL</t>
+          <t>FCAP</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ACNB</t>
+          <t>FRME</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>BOKF</t>
+          <t>ADUS</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>OSPN</t>
+          <t>ASBH</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>ACU</t>
+          <t>ASO</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CASY</t>
+          <t>DGII</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>REGN</t>
+          <t>IBG</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>ADP</t>
+          <t>ALRS</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CHDN</t>
+          <t>AUDC</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>SHOE</t>
+          <t>DPZ</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>ADPT</t>
+          <t>IMCR</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CLRO</t>
+          <t>AVAH</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>ADSK</t>
+          <t>ESTA</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>COLL</t>
+          <t>JRVR</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>TOMZ</t>
+          <t>AWR</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>ADUS</t>
+          <t>EVER</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>AEP</t>
+          <t>NYAX</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>CRNT</t>
+          <t>ANDG</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>AFRI</t>
+          <t>PECO</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>CWST</t>
+          <t>API</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>AGYS</t>
+          <t>AXIN</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>DPZ</t>
+          <t>PLUR</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>ALKS</t>
+          <t>AROW</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>EJH</t>
+          <t>BHRB</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>ALLT</t>
+          <t>GAUZ</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>ESTA</t>
+          <t>PRTA</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>ALRS</t>
+          <t>ATLCL</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>EVER</t>
+          <t>INSG</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>AMGN</t>
+          <t>ATLCZ</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>EXTR</t>
+          <t>BL</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>AMRX</t>
+          <t>INTJ</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>ANIK</t>
+          <t>RDCM</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>APA</t>
+          <t>ATR</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IDN</t>
+          <t>BLKB</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>API</t>
+          <t>JLHL</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>IMCR</t>
+          <t>SBCF</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>INSG</t>
+          <t>AUPH</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>AROW</t>
+          <t>BMBL</t>
         </is>
       </c>
     </row>
@@ -818,2499 +818,1974 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>ARQT</t>
+          <t>BMRC</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LMAT</t>
+          <t>NBIX</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>ARX</t>
+          <t>TCBK</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>LWAY</t>
+          <t>BANF</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>ASBH</t>
+          <t>BOLT</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>MGEE</t>
+          <t>NBTX</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ASND</t>
+          <t>TCX</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>NBIX</t>
+          <t>BBCP</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>ATLCL</t>
+          <t>BOW</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>NBN</t>
+          <t>NXST</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>ATLCZ</t>
+          <t>YORW</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>NXST</t>
+          <t>BR</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>ATR</t>
+          <t>BFST</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>NYAX</t>
+          <t>BIII</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>AUDC</t>
+          <t>BUUU</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>OFIX</t>
+          <t>BMGL</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>AUPH</t>
+          <t>CARL</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>PATK</t>
+          <t>PRPL</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>AVBC</t>
+          <t>BOBS</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>PAYX</t>
+          <t>CATY</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>AVBH</t>
+          <t>PWRL</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>PECO</t>
+          <t>BOOM</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>AWR</t>
+          <t>CBRL</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>AXGN</t>
+          <t>QNST</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>PLUR</t>
+          <t>BSIN</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>PRTA</t>
+          <t>CENT</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>BBCP</t>
+          <t>CEPO</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>QQQX</t>
+          <t>SMBC</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>RARE</t>
+          <t>BWFG</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>BFST</t>
+          <t>CERT</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>RDCM</t>
+          <t>TCMD</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>BHRB</t>
+          <t>CHRD</t>
         </is>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>BIIB</t>
+          <t>CBC</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>SMBC</t>
+          <t>CING</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>BL</t>
+          <t>CBU</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>SOLS</t>
+          <t>CIVB</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>BLKB</t>
+          <t>CCID</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>TCBK</t>
+          <t>COFS</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>BMGL</t>
+          <t>CCNE</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>TCX</t>
+          <t>CDLR</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>BMRC</t>
+          <t>CRVL</t>
         </is>
       </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>VMRK</t>
+          <t>CDNA</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>BOOM</t>
+          <t>CVBF</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>YORW</t>
+          <t>CENTA</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>BOW</t>
+          <t>CZNC</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>BR</t>
+          <t>CGNT</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>BSBK</t>
+          <t>DCOM</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>BSIN</t>
+          <t>CHCO</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>BSP</t>
+          <t>DMAA</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>BUUU</t>
+          <t>DORM</t>
         </is>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>BVC</t>
+          <t>CHOW</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>BVFL</t>
+          <t>ECBK</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>BWFG</t>
+          <t>CHPGU</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>BZ</t>
+          <t>EFSC</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>CARL</t>
+          <t>CIGI</t>
         </is>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>CATY</t>
+          <t>EML</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>CBC</t>
+          <t>CINF</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>CBK</t>
+          <t>ENGS</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>CBU</t>
+          <t>COAG</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>CCEP</t>
+          <t>ENTX</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>CCID</t>
+          <t>EPSN</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>CCNE</t>
+          <t>ESQ</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>CDLR</t>
+          <t>EWBC</t>
         </is>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>CENT</t>
+          <t>CPSS</t>
         </is>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>CENTA</t>
+          <t>FA</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>CERT</t>
+          <t>FBLA</t>
         </is>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>CGNT</t>
+          <t>CZFS</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>CHCO</t>
+          <t>FBNC</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>CHKP</t>
+          <t>CZWI</t>
         </is>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>CHRD</t>
+          <t>FCCO</t>
         </is>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>CIGI</t>
+          <t>FCNCA</t>
         </is>
       </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>CINF</t>
+          <t>DMRC</t>
         </is>
       </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>CING</t>
+          <t>FFTT</t>
         </is>
       </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>CIVB</t>
+          <t>DOX</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>CLGN</t>
+          <t>FGCPP</t>
         </is>
       </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>CME</t>
+          <t>DUKU</t>
         </is>
       </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>COAG</t>
+          <t>FIZZ</t>
         </is>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>COFS</t>
+          <t>FNLC</t>
         </is>
       </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>COLM</t>
+          <t>EDHL</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>COST</t>
+          <t>FSSL</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>CRAI</t>
+          <t>FTDR</t>
         </is>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>CRVL</t>
+          <t>ERIE</t>
         </is>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>CTAS</t>
+          <t>FULT</t>
         </is>
       </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>CVBF</t>
+          <t>GAINI</t>
         </is>
       </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>CZFS</t>
+          <t>GIBO</t>
         </is>
       </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>CZNC</t>
+          <t>GSBC</t>
         </is>
       </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>CZWI</t>
+          <t>EXPO</t>
         </is>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>DCBO</t>
+          <t>FBIZ</t>
         </is>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>DCOM</t>
+          <t>HBT</t>
         </is>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>DGII</t>
+          <t>FLYW</t>
         </is>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>DLTR</t>
+          <t>HCKT</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>DMAA</t>
+          <t>FMNB</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>DMII</t>
+          <t>HELE</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>DORM</t>
+          <t>FRAF</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>DOX</t>
+          <t>HFWA</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>FRHC</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>DUKU</t>
+          <t>HQY</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>EFSC</t>
+          <t>FSBC</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>ENGS</t>
+          <t>HUIZ</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>EPSN</t>
+          <t>FSV</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>ERIC</t>
+          <t>HURN</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>ERIE</t>
+          <t>FWRD</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>ESQ</t>
+          <t>HWBK</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>EVRG</t>
+          <t>GAING</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>EWBC</t>
+          <t>HWKN</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>EXLS</t>
+          <t>GCT</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>EXPO</t>
+          <t>IIIV</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>FA</t>
+          <t>GDYN</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>FANG</t>
+          <t>INDB</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>FBNC</t>
+          <t>INVE</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>FCBM</t>
+          <t>IOSP</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>FCCO</t>
+          <t>IRON</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>FCNCA</t>
+          <t>ITRI</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>FDBC</t>
+          <t>HAFC</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>FGBI</t>
+          <t>JAKK</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>FIZZ</t>
+          <t>HBIO</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>FMAO</t>
+          <t>JANX</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>FNLC</t>
+          <t>HBNC</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>FRAF</t>
+          <t>JJSF</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>FRBA</t>
+          <t>HOFT</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>FRD</t>
+          <t>JVA</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>FRHC</t>
+          <t>KBON</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>FRME</t>
+          <t>KELYA</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>FSBC</t>
+          <t>ICON</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>FSSL</t>
+          <t>KFII</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>FTDR</t>
+          <t>ICUI</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>FULT</t>
+          <t>KGEI</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>FUNC</t>
+          <t>IDXX</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>GAING</t>
+          <t>KINS</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>GCBC</t>
+          <t>III</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>GCL</t>
+          <t>KMTS</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>GCT</t>
+          <t>INTG</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>GIBO</t>
+          <t>KRRO</t>
         </is>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>GO</t>
+          <t>LCNB</t>
         </is>
       </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>GRFS</t>
+          <t>INVA</t>
         </is>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>GSAT</t>
+          <t>IPAR</t>
         </is>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>GSBC</t>
+          <t>LKFN</t>
         </is>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>GTLB</t>
+          <t>IRTC</t>
         </is>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>HAFC</t>
+          <t>LLYVA</t>
         </is>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>HALO</t>
+          <t>LLYVK</t>
         </is>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>HAS</t>
+          <t>JKHY</t>
         </is>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>HBIO</t>
+          <t>LMRI</t>
         </is>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>HBNC</t>
+          <t>LSBK</t>
         </is>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>HCKT</t>
+          <t>LZ</t>
         </is>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>HELE</t>
+          <t>MIDD</t>
         </is>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>HFWA</t>
+          <t>KYMR</t>
         </is>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>HON</t>
+          <t>MKTW</t>
         </is>
       </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
         <is>
-          <t>HTHT</t>
+          <t>LEGH</t>
         </is>
       </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
         <is>
-          <t>HURN</t>
+          <t>MOBI</t>
         </is>
       </c>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
         <is>
-          <t>HWBK</t>
+          <t>MORN</t>
         </is>
       </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
         <is>
-          <t>HWKN</t>
+          <t>LGND</t>
         </is>
       </c>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>ICFI</t>
+          <t>MRVI</t>
         </is>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>IDXX</t>
+          <t>MSBI</t>
         </is>
       </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
         <is>
-          <t>III</t>
+          <t>MYFW</t>
         </is>
       </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
         <is>
-          <t>IIIV</t>
+          <t>NBTB</t>
         </is>
       </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
         <is>
-          <t>INTU</t>
+          <t>MASS</t>
         </is>
       </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
         <is>
-          <t>INVA</t>
+          <t>NPAC</t>
         </is>
       </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
         <is>
-          <t>IOSP</t>
+          <t>MAYS</t>
         </is>
       </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
         <is>
-          <t>IPAR</t>
+          <t>NRC</t>
         </is>
       </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
         <is>
-          <t>IRON</t>
+          <t>MEOH</t>
         </is>
       </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
         <is>
-          <t>ISBA</t>
+          <t>MGYR</t>
         </is>
       </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
         <is>
-          <t>ISRG</t>
+          <t>MICC</t>
         </is>
       </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
         <is>
-          <t>ITRI</t>
+          <t>NWBI</t>
         </is>
       </c>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
         <is>
-          <t>JAKK</t>
+          <t>MKTX</t>
         </is>
       </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
         <is>
-          <t>JANX</t>
+          <t>NWFL</t>
         </is>
       </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
         <is>
-          <t>JJSF</t>
+          <t>OCTV</t>
         </is>
       </c>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
         <is>
-          <t>JKHY</t>
+          <t>OLED</t>
         </is>
       </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
         <is>
-          <t>JOUT</t>
+          <t>MSEX</t>
         </is>
       </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
         <is>
-          <t>JVA</t>
+          <t>OMAB</t>
         </is>
       </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
         <is>
-          <t>KARO</t>
+          <t>MZTI</t>
         </is>
       </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
         <is>
-          <t>KELYA</t>
+          <t>OPLN</t>
         </is>
       </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
         <is>
-          <t>KGEI</t>
+          <t>ORKA</t>
         </is>
       </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
         <is>
-          <t>KINS</t>
+          <t>NMFCZ</t>
         </is>
       </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
         <is>
-          <t>KMRK</t>
+          <t>OVLY</t>
         </is>
       </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
         <is>
-          <t>KROS</t>
+          <t>NOVTU</t>
         </is>
       </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
         <is>
-          <t>LBRX</t>
+          <t>NSLRL</t>
         </is>
       </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
         <is>
-          <t>LCNB</t>
+          <t>PBFS</t>
         </is>
       </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
         <is>
-          <t>LEGH</t>
+          <t>PCB</t>
         </is>
       </c>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
         <is>
-          <t>LEGN</t>
+          <t>NWE</t>
         </is>
       </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
         <is>
-          <t>LGND</t>
+          <t>PFXNZ</t>
         </is>
       </c>
     </row>
     <row r="238">
       <c r="A238" t="inlineStr">
         <is>
-          <t>LIFE</t>
+          <t>OBT</t>
         </is>
       </c>
     </row>
     <row r="239">
       <c r="A239" t="inlineStr">
         <is>
-          <t>LIN</t>
+          <t>PLGO</t>
         </is>
       </c>
     </row>
     <row r="240">
       <c r="A240" t="inlineStr">
         <is>
-          <t>LKFN</t>
+          <t>PLMR</t>
         </is>
       </c>
     </row>
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>LKFT</t>
+          <t>ORRF</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>LLYVA</t>
+          <t>PMTR</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>LLYVK</t>
+          <t>OSG</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>LMRI</t>
+          <t>PNRG</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>LOVE</t>
+          <t>OSPN</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>LSBK</t>
+          <t>POOL</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>LYEL</t>
+          <t>PRGS</t>
         </is>
       </c>
     </row>
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>LZ</t>
+          <t>PACH</t>
         </is>
       </c>
     </row>
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>MANH</t>
+          <t>PAHC</t>
         </is>
       </c>
     </row>
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>MAR</t>
+          <t>PYPD</t>
         </is>
       </c>
     </row>
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>MASS</t>
+          <t>PCTY</t>
         </is>
       </c>
     </row>
     <row r="252">
       <c r="A252" t="inlineStr">
         <is>
-          <t>MAZE</t>
+          <t>QCRH</t>
         </is>
       </c>
     </row>
     <row r="253">
       <c r="A253" t="inlineStr">
         <is>
-          <t>MBWM</t>
+          <t>PDLB</t>
         </is>
       </c>
     </row>
     <row r="254">
       <c r="A254" t="inlineStr">
         <is>
-          <t>MCHX</t>
+          <t>QNBC</t>
         </is>
       </c>
     </row>
     <row r="255">
       <c r="A255" t="inlineStr">
         <is>
-          <t>MGPI</t>
+          <t>PEBO</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" t="inlineStr">
         <is>
-          <t>MGYR</t>
+          <t>RCBC</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" t="inlineStr">
         <is>
-          <t>MICC</t>
+          <t>PGC</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" t="inlineStr">
         <is>
-          <t>MKTX</t>
+          <t>REF</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" t="inlineStr">
         <is>
-          <t>MORN</t>
+          <t>PGNY</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" t="inlineStr">
         <is>
-          <t>MRSH</t>
+          <t>RELL</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" t="inlineStr">
         <is>
-          <t>MRVI</t>
+          <t>PLBY</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" t="inlineStr">
         <is>
-          <t>MSBI</t>
+          <t>REYN</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" t="inlineStr">
         <is>
-          <t>MSEX</t>
+          <t>PNTG</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" t="inlineStr">
         <is>
-          <t>MTEX</t>
+          <t>SAGT</t>
         </is>
       </c>
     </row>
     <row r="265">
       <c r="A265" t="inlineStr">
         <is>
-          <t>MYFW</t>
+          <t>PPLC</t>
         </is>
       </c>
     </row>
     <row r="266">
       <c r="A266" t="inlineStr">
         <is>
-          <t>MZTI</t>
+          <t>SBAC</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" t="inlineStr">
         <is>
-          <t>NBTB</t>
+          <t>SGP</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" t="inlineStr">
         <is>
-          <t>NBTX</t>
+          <t>RDWR</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" t="inlineStr">
         <is>
-          <t>NDAQ</t>
+          <t>SHPH</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" t="inlineStr">
         <is>
-          <t>NRC</t>
+          <t>SIGI</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" t="inlineStr">
         <is>
-          <t>NRDS</t>
+          <t>REGN</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" t="inlineStr">
         <is>
-          <t>NRIX</t>
+          <t>SKYA</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" t="inlineStr">
         <is>
-          <t>NTLA</t>
+          <t>SLDE</t>
         </is>
       </c>
     </row>
     <row r="274">
       <c r="A274" t="inlineStr">
         <is>
-          <t>NWBI</t>
+          <t>RGCO</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" t="inlineStr">
         <is>
-          <t>NWE</t>
+          <t>SNES</t>
         </is>
       </c>
     </row>
     <row r="276">
       <c r="A276" t="inlineStr">
         <is>
-          <t>NWFL</t>
+          <t>ROOT</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" t="inlineStr">
         <is>
-          <t>OBT</t>
+          <t>SOMN</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" t="inlineStr">
         <is>
-          <t>OCTV</t>
+          <t>SORA</t>
         </is>
       </c>
     </row>
     <row r="279">
       <c r="A279" t="inlineStr">
         <is>
-          <t>OIO</t>
+          <t>SRCE</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
         <is>
-          <t>OLED</t>
+          <t>RRBI</t>
         </is>
       </c>
     </row>
     <row r="281">
       <c r="A281" t="inlineStr">
         <is>
-          <t>OPK</t>
+          <t>SRPT</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" t="inlineStr">
         <is>
-          <t>OPLN</t>
+          <t>SRZN</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" t="inlineStr">
         <is>
-          <t>ORRF</t>
+          <t>RYZ</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" t="inlineStr">
         <is>
-          <t>OSW</t>
+          <t>SYRE</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" t="inlineStr">
         <is>
-          <t>OVLY</t>
+          <t>SAIC</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" t="inlineStr">
         <is>
-          <t>OZK</t>
+          <t>UTHR</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" t="inlineStr">
         <is>
-          <t>PCB</t>
+          <t>VIR</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" t="inlineStr">
         <is>
-          <t>PCTY</t>
+          <t>SCHL</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" t="inlineStr">
         <is>
-          <t>PDLB</t>
+          <t>WHK</t>
         </is>
       </c>
     </row>
     <row r="290">
       <c r="A290" t="inlineStr">
         <is>
-          <t>PEBO</t>
+          <t>YSWY</t>
         </is>
       </c>
     </row>
     <row r="291">
       <c r="A291" t="inlineStr">
         <is>
-          <t>PFIS</t>
+          <t>SEZL</t>
         </is>
       </c>
     </row>
     <row r="292">
       <c r="A292" t="inlineStr">
         <is>
-          <t>PFXNZ</t>
+          <t>SHOE</t>
         </is>
       </c>
     </row>
     <row r="293">
       <c r="A293" t="inlineStr">
         <is>
-          <t>PGC</t>
+          <t>SLAB</t>
         </is>
       </c>
     </row>
     <row r="294">
       <c r="A294" t="inlineStr">
         <is>
-          <t>PGNY</t>
+          <t>SNFCA</t>
         </is>
       </c>
     </row>
     <row r="295">
       <c r="A295" t="inlineStr">
         <is>
-          <t>PLBC</t>
+          <t>SWIM</t>
         </is>
       </c>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
         <is>
-          <t>PLGO</t>
+          <t>SYNA</t>
         </is>
       </c>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
         <is>
-          <t>PLMR</t>
+          <t>TGTX</t>
         </is>
       </c>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
         <is>
-          <t>PNFP</t>
+          <t>TLS</t>
         </is>
       </c>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
         <is>
-          <t>PNTG</t>
+          <t>TOMZ</t>
         </is>
       </c>
     </row>
     <row r="300">
       <c r="A300" t="inlineStr">
         <is>
-          <t>PODD</t>
+          <t>TRGSU</t>
         </is>
       </c>
     </row>
     <row r="301">
       <c r="A301" t="inlineStr">
         <is>
-          <t>POOL</t>
+          <t>TVACU</t>
         </is>
       </c>
     </row>
     <row r="302">
       <c r="A302" t="inlineStr">
         <is>
-          <t>PRGS</t>
+          <t>WTW</t>
         </is>
       </c>
     </row>
     <row r="303">
       <c r="A303" t="inlineStr">
         <is>
-          <t>PTC</t>
+          <t>XZO</t>
         </is>
       </c>
     </row>
     <row r="304">
       <c r="A304" t="inlineStr">
         <is>
-          <t>PTEN</t>
+          <t>INM</t>
         </is>
       </c>
     </row>
     <row r="305">
       <c r="A305" t="inlineStr">
         <is>
-          <t>PTLE</t>
+          <t>SPCB</t>
         </is>
       </c>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
         <is>
-          <t>PTLO</t>
+          <t>AVBC</t>
         </is>
       </c>
     </row>
     <row r="307">
       <c r="A307" t="inlineStr">
         <is>
-          <t>PWRL</t>
+          <t>STFS</t>
         </is>
       </c>
     </row>
     <row r="308">
       <c r="A308" t="inlineStr">
         <is>
-          <t>PYPD</t>
+          <t>NORD</t>
         </is>
       </c>
     </row>
     <row r="309">
       <c r="A309" t="inlineStr">
         <is>
-          <t>QCRH</t>
+          <t>BETR</t>
         </is>
       </c>
     </row>
     <row r="310">
       <c r="A310" t="inlineStr">
         <is>
-          <t>QNBC</t>
+          <t>RIBBU</t>
         </is>
       </c>
     </row>
     <row r="311">
       <c r="A311" t="inlineStr">
         <is>
-          <t>RCBC</t>
+          <t>DOO</t>
         </is>
       </c>
     </row>
     <row r="312">
       <c r="A312" t="inlineStr">
         <is>
-          <t>RDWR</t>
+          <t>EFOI</t>
         </is>
       </c>
     </row>
     <row r="313">
       <c r="A313" t="inlineStr">
         <is>
-          <t>REF</t>
+          <t>BRCB</t>
         </is>
       </c>
     </row>
     <row r="314">
       <c r="A314" t="inlineStr">
         <is>
-          <t>RELL</t>
+          <t>FIVE</t>
         </is>
       </c>
     </row>
     <row r="315">
       <c r="A315" t="inlineStr">
         <is>
-          <t>REYN</t>
+          <t>OPRT</t>
         </is>
       </c>
     </row>
     <row r="316">
       <c r="A316" t="inlineStr">
         <is>
-          <t>RIGL</t>
+          <t>RICK</t>
         </is>
       </c>
     </row>
     <row r="317">
       <c r="A317" t="inlineStr">
         <is>
-          <t>RMBI</t>
+          <t>ATEX</t>
         </is>
       </c>
     </row>
     <row r="318">
       <c r="A318" t="inlineStr">
         <is>
-          <t>ROOT</t>
+          <t>HYNE</t>
         </is>
       </c>
     </row>
     <row r="319">
       <c r="A319" t="inlineStr">
         <is>
-          <t>ROP</t>
+          <t>RIGL</t>
         </is>
       </c>
     </row>
     <row r="320">
       <c r="A320" t="inlineStr">
         <is>
-          <t>RPRX</t>
+          <t>ATGL</t>
         </is>
       </c>
     </row>
     <row r="321">
       <c r="A321" t="inlineStr">
         <is>
-          <t>RRBI</t>
+          <t>STAA</t>
         </is>
       </c>
     </row>
     <row r="322">
       <c r="A322" t="inlineStr">
         <is>
-          <t>RYZ</t>
+          <t>XFOR</t>
         </is>
       </c>
     </row>
     <row r="323">
       <c r="A323" t="inlineStr">
         <is>
-          <t>SAFT</t>
+          <t>PHAR</t>
         </is>
       </c>
     </row>
     <row r="324">
       <c r="A324" t="inlineStr">
         <is>
-          <t>SAGT</t>
+          <t>KXIN</t>
         </is>
       </c>
     </row>
     <row r="325">
       <c r="A325" t="inlineStr">
         <is>
-          <t>SAIC</t>
+          <t>CHSN</t>
         </is>
       </c>
     </row>
     <row r="326">
       <c r="A326" t="inlineStr">
         <is>
-          <t>SBAC</t>
+          <t>CLAR</t>
         </is>
       </c>
     </row>
     <row r="327">
       <c r="A327" t="inlineStr">
         <is>
-          <t>SCAG</t>
+          <t>RJET</t>
         </is>
       </c>
     </row>
     <row r="328">
       <c r="A328" t="inlineStr">
         <is>
-          <t>SCHL</t>
+          <t>FGBI</t>
         </is>
       </c>
     </row>
     <row r="329">
       <c r="A329" t="inlineStr">
         <is>
-          <t>SDGR</t>
+          <t>GRFS</t>
         </is>
       </c>
     </row>
     <row r="330">
       <c r="A330" t="inlineStr">
         <is>
-          <t>SFNC</t>
+          <t>CTKB</t>
         </is>
       </c>
     </row>
     <row r="331">
       <c r="A331" t="inlineStr">
         <is>
-          <t>SGP</t>
+          <t>XNCR</t>
         </is>
       </c>
     </row>
     <row r="332">
       <c r="A332" t="inlineStr">
         <is>
-          <t>SHPH</t>
+          <t>IMC</t>
         </is>
       </c>
     </row>
     <row r="333">
       <c r="A333" t="inlineStr">
         <is>
-          <t>SIGI</t>
+          <t>DHCNL</t>
         </is>
       </c>
     </row>
     <row r="334">
       <c r="A334" t="inlineStr">
         <is>
-          <t>SNES</t>
+          <t>HLP</t>
         </is>
       </c>
     </row>
     <row r="335">
       <c r="A335" t="inlineStr">
         <is>
-          <t>SNFCA</t>
+          <t>KPLT</t>
         </is>
       </c>
     </row>
     <row r="336">
       <c r="A336" t="inlineStr">
         <is>
-          <t>SOMN</t>
+          <t>DIBS</t>
         </is>
       </c>
     </row>
     <row r="337">
       <c r="A337" t="inlineStr">
         <is>
-          <t>SRCE</t>
+          <t>ATER</t>
         </is>
       </c>
     </row>
     <row r="338">
       <c r="A338" t="inlineStr">
         <is>
-          <t>SRPT</t>
+          <t>KOD</t>
         </is>
       </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
         <is>
-          <t>SRZN</t>
-        </is>
-      </c>
-    </row>
-    <row r="340">
-      <c r="A340" t="inlineStr">
-        <is>
-          <t>SYNA</t>
-        </is>
-      </c>
-    </row>
-    <row r="341">
-      <c r="A341" t="inlineStr">
-        <is>
-          <t>SYRE</t>
-        </is>
-      </c>
-    </row>
-    <row r="342">
-      <c r="A342" t="inlineStr">
-        <is>
-          <t>TACT</t>
-        </is>
-      </c>
-    </row>
-    <row r="343">
-      <c r="A343" t="inlineStr">
-        <is>
-          <t>TCMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="344">
-      <c r="A344" t="inlineStr">
-        <is>
-          <t>TGTX</t>
-        </is>
-      </c>
-    </row>
-    <row r="345">
-      <c r="A345" t="inlineStr">
-        <is>
-          <t>THFF</t>
-        </is>
-      </c>
-    </row>
-    <row r="346">
-      <c r="A346" t="inlineStr">
-        <is>
-          <t>TILE</t>
-        </is>
-      </c>
-    </row>
-    <row r="347">
-      <c r="A347" t="inlineStr">
-        <is>
-          <t>TLS</t>
-        </is>
-      </c>
-    </row>
-    <row r="348">
-      <c r="A348" t="inlineStr">
-        <is>
-          <t>TRI</t>
-        </is>
-      </c>
-    </row>
-    <row r="349">
-      <c r="A349" t="inlineStr">
-        <is>
-          <t>TRMB</t>
-        </is>
-      </c>
-    </row>
-    <row r="350">
-      <c r="A350" t="inlineStr">
-        <is>
-          <t>TW</t>
-        </is>
-      </c>
-    </row>
-    <row r="351">
-      <c r="A351" t="inlineStr">
-        <is>
-          <t>UTHR</t>
-        </is>
-      </c>
-    </row>
-    <row r="352">
-      <c r="A352" t="inlineStr">
-        <is>
-          <t>VIR</t>
-        </is>
-      </c>
-    </row>
-    <row r="353">
-      <c r="A353" t="inlineStr">
-        <is>
-          <t>WCCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="354">
-      <c r="A354" t="inlineStr">
-        <is>
-          <t>WHK</t>
-        </is>
-      </c>
-    </row>
-    <row r="355">
-      <c r="A355" t="inlineStr">
-        <is>
-          <t>WTW</t>
-        </is>
-      </c>
-    </row>
-    <row r="356">
-      <c r="A356" t="inlineStr">
-        <is>
-          <t>YSWY</t>
-        </is>
-      </c>
-    </row>
-    <row r="357">
-      <c r="A357" t="inlineStr">
-        <is>
-          <t>DMRC</t>
-        </is>
-      </c>
-    </row>
-    <row r="358">
-      <c r="A358" t="inlineStr">
-        <is>
-          <t>EFOI</t>
-        </is>
-      </c>
-    </row>
-    <row r="359">
-      <c r="A359" t="inlineStr">
-        <is>
-          <t>STAA</t>
-        </is>
-      </c>
-    </row>
-    <row r="360">
-      <c r="A360" t="inlineStr">
-        <is>
-          <t>BETR</t>
-        </is>
-      </c>
-    </row>
-    <row r="361">
-      <c r="A361" t="inlineStr">
-        <is>
-          <t>CLAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="362">
-      <c r="A362" t="inlineStr">
-        <is>
-          <t>RIBBU</t>
-        </is>
-      </c>
-    </row>
-    <row r="363">
-      <c r="A363" t="inlineStr">
-        <is>
-          <t>FIVE</t>
-        </is>
-      </c>
-    </row>
-    <row r="364">
-      <c r="A364" t="inlineStr">
-        <is>
-          <t>KPLT</t>
-        </is>
-      </c>
-    </row>
-    <row r="365">
-      <c r="A365" t="inlineStr">
-        <is>
-          <t>DIBS</t>
-        </is>
-      </c>
-    </row>
-    <row r="366">
-      <c r="A366" t="inlineStr">
-        <is>
-          <t>GNSS</t>
-        </is>
-      </c>
-    </row>
-    <row r="367">
-      <c r="A367" t="inlineStr">
-        <is>
-          <t>SWIM</t>
-        </is>
-      </c>
-    </row>
-    <row r="368">
-      <c r="A368" t="inlineStr">
-        <is>
-          <t>HLP</t>
-        </is>
-      </c>
-    </row>
-    <row r="369">
-      <c r="A369" t="inlineStr">
-        <is>
-          <t>OPRT</t>
-        </is>
-      </c>
-    </row>
-    <row r="370">
-      <c r="A370" t="inlineStr">
-        <is>
-          <t>DOO</t>
-        </is>
-      </c>
-    </row>
-    <row r="371">
-      <c r="A371" t="inlineStr">
-        <is>
-          <t>APOG</t>
-        </is>
-      </c>
-    </row>
-    <row r="372">
-      <c r="A372" t="inlineStr">
-        <is>
-          <t>ATEX</t>
-        </is>
-      </c>
-    </row>
-    <row r="373">
-      <c r="A373" t="inlineStr">
-        <is>
-          <t>SGRY</t>
-        </is>
-      </c>
-    </row>
-    <row r="374">
-      <c r="A374" t="inlineStr">
-        <is>
-          <t>PRPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="375">
-      <c r="A375" t="inlineStr">
-        <is>
-          <t>ORKA</t>
-        </is>
-      </c>
-    </row>
-    <row r="376">
-      <c r="A376" t="inlineStr">
-        <is>
-          <t>IBG</t>
-        </is>
-      </c>
-    </row>
-    <row r="377">
-      <c r="A377" t="inlineStr">
-        <is>
-          <t>TMCI</t>
-        </is>
-      </c>
-    </row>
-    <row r="378">
-      <c r="A378" t="inlineStr">
-        <is>
-          <t>ATGL</t>
-        </is>
-      </c>
-    </row>
-    <row r="379">
-      <c r="A379" t="inlineStr">
-        <is>
-          <t>ICON</t>
-        </is>
-      </c>
-    </row>
-    <row r="380">
-      <c r="A380" t="inlineStr">
-        <is>
-          <t>GLSI</t>
-        </is>
-      </c>
-    </row>
-    <row r="381">
-      <c r="A381" t="inlineStr">
-        <is>
-          <t>CTKB</t>
-        </is>
-      </c>
-    </row>
-    <row r="382">
-      <c r="A382" t="inlineStr">
-        <is>
           <t>LUNG</t>
-        </is>
-      </c>
-    </row>
-    <row r="383">
-      <c r="A383" t="inlineStr">
-        <is>
-          <t>KRRO</t>
-        </is>
-      </c>
-    </row>
-    <row r="384">
-      <c r="A384" t="inlineStr">
-        <is>
-          <t>CHSN</t>
-        </is>
-      </c>
-    </row>
-    <row r="385">
-      <c r="A385" t="inlineStr">
-        <is>
-          <t>LVO</t>
-        </is>
-      </c>
-    </row>
-    <row r="386">
-      <c r="A386" t="inlineStr">
-        <is>
-          <t>SGHT</t>
-        </is>
-      </c>
-    </row>
-    <row r="387">
-      <c r="A387" t="inlineStr">
-        <is>
-          <t>REPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="388">
-      <c r="A388" t="inlineStr">
-        <is>
-          <t>AVPT</t>
-        </is>
-      </c>
-    </row>
-    <row r="389">
-      <c r="A389" t="inlineStr">
-        <is>
-          <t>KXIN</t>
-        </is>
-      </c>
-    </row>
-    <row r="390">
-      <c r="A390" t="inlineStr">
-        <is>
-          <t>ATER</t>
-        </is>
-      </c>
-    </row>
-    <row r="391">
-      <c r="A391" t="inlineStr">
-        <is>
-          <t>PHAR</t>
-        </is>
-      </c>
-    </row>
-    <row r="392">
-      <c r="A392" t="inlineStr">
-        <is>
-          <t>ALRM</t>
-        </is>
-      </c>
-    </row>
-    <row r="393">
-      <c r="A393" t="inlineStr">
-        <is>
-          <t>TRMD</t>
-        </is>
-      </c>
-    </row>
-    <row r="394">
-      <c r="A394" t="inlineStr">
-        <is>
-          <t>BRCB</t>
-        </is>
-      </c>
-    </row>
-    <row r="395">
-      <c r="A395" t="inlineStr">
-        <is>
-          <t>RJET</t>
-        </is>
-      </c>
-    </row>
-    <row r="396">
-      <c r="A396" t="inlineStr">
-        <is>
-          <t>KVHI</t>
-        </is>
-      </c>
-    </row>
-    <row r="397">
-      <c r="A397" t="inlineStr">
-        <is>
-          <t>PNRG</t>
-        </is>
-      </c>
-    </row>
-    <row r="398">
-      <c r="A398" t="inlineStr">
-        <is>
-          <t>HYNE</t>
-        </is>
-      </c>
-    </row>
-    <row r="399">
-      <c r="A399" t="inlineStr">
-        <is>
-          <t>SEPN</t>
-        </is>
-      </c>
-    </row>
-    <row r="400">
-      <c r="A400" t="inlineStr">
-        <is>
-          <t>MLTX</t>
-        </is>
-      </c>
-    </row>
-    <row r="401">
-      <c r="A401" t="inlineStr">
-        <is>
-          <t>CHMG</t>
-        </is>
-      </c>
-    </row>
-    <row r="402">
-      <c r="A402" t="inlineStr">
-        <is>
-          <t>IMC</t>
-        </is>
-      </c>
-    </row>
-    <row r="403">
-      <c r="A403" t="inlineStr">
-        <is>
-          <t>KOD</t>
-        </is>
-      </c>
-    </row>
-    <row r="404">
-      <c r="A404" t="inlineStr">
-        <is>
-          <t>RCEL</t>
-        </is>
-      </c>
-    </row>
-    <row r="405">
-      <c r="A405" t="inlineStr">
-        <is>
-          <t>MOBI</t>
-        </is>
-      </c>
-    </row>
-    <row r="406">
-      <c r="A406" t="inlineStr">
-        <is>
-          <t>LFST</t>
-        </is>
-      </c>
-    </row>
-    <row r="407">
-      <c r="A407" t="inlineStr">
-        <is>
-          <t>ADMA</t>
-        </is>
-      </c>
-    </row>
-    <row r="408">
-      <c r="A408" t="inlineStr">
-        <is>
-          <t>FFTT</t>
-        </is>
-      </c>
-    </row>
-    <row r="409">
-      <c r="A409" t="inlineStr">
-        <is>
-          <t>XNCR</t>
-        </is>
-      </c>
-    </row>
-    <row r="410">
-      <c r="A410" t="inlineStr">
-        <is>
-          <t>JLHL</t>
-        </is>
-      </c>
-    </row>
-    <row r="411">
-      <c r="A411" t="inlineStr">
-        <is>
-          <t>STFS</t>
-        </is>
-      </c>
-    </row>
-    <row r="412">
-      <c r="A412" t="inlineStr">
-        <is>
-          <t>MYGN</t>
-        </is>
-      </c>
-    </row>
-    <row r="413">
-      <c r="A413" t="inlineStr">
-        <is>
-          <t>MANE</t>
-        </is>
-      </c>
-    </row>
-    <row r="414">
-      <c r="A414" t="inlineStr">
-        <is>
-          <t>SLN</t>
         </is>
       </c>
     </row>

</xml_diff>